<commit_message>
Raise Scale price and year-2 Sprint volume
Scale goes from R$ 18.997 to R$ 29.997 (6x R$ 4.999,50) and the Sprint
is also sold outside the Core base in year 2 (54 instead of 27). VPL at
24% a.a. rises from R$ 84,9 mil to R$ 126,1 mil; break-even (month 6)
and runway (4 months) are unchanged. Workbook still only fills the gray
cells; the form and the calculation memo are regenerated from one model.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016kLWp3PkVdryYcjkVkag3m
</commit_message>
<xml_diff>
--- a/precept-financeiro/Memoria_de_Calculo_Precept.xlsx
+++ b/precept-financeiro/Memoria_de_Calculo_Precept.xlsx
@@ -345,13 +345,13 @@
     <t xml:space="preserve">Precept Sprint – imersão de 7 dias (R$, à vista)</t>
   </si>
   <si>
-    <t xml:space="preserve">Preço definido pelo grupo: planejamento estratégico e tático em 7 dias imersivos.</t>
+    <t xml:space="preserve">Preço definido pelo grupo: planejamento estratégico e tático em 7 dias imersivos. No ano 2, também vendido para escritórios fora da base Core (4 a 5 por mês), no modelo das imersões da G4.</t>
   </si>
   <si>
     <t xml:space="preserve">Precept Scale – implementação (R$ por projeto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Preço definido pelo grupo: implementação e acompanhamento dos 6 pilares.</t>
+    <t xml:space="preserve">Preço proposto para o início da operação: 3× o Sprint e ~R$ 5 mil/mês por 6 meses, abaixo de consultorias de gestão para PMEs (R$ 8–15 mil/mês). Cerca de 1% a 3% do faturamento anual de um escritório de R$ 1–4 mi.</t>
   </si>
   <si>
     <t xml:space="preserve">Parcelas do Scale (meses de projeto)</t>
@@ -2037,7 +2037,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
         <v>39</v>
       </c>
@@ -2048,12 +2048,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
         <v>41</v>
       </c>
       <c r="B10" s="12" t="n">
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>42</v>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="B12" s="15" t="n">
         <f aca="false">B10/B11</f>
-        <v>3166.16666666667</v>
+        <v>4999.5</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>46</v>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B71" s="28" t="n">
         <f aca="false">'VPL e TIR'!B38</f>
-        <v>84862.163322548</v>
+        <v>126073.58365125</v>
       </c>
       <c r="C71" s="13" t="s">
         <v>138</v>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B72" s="29" t="n">
         <f aca="false">'VPL e TIR'!B40</f>
-        <v>0.795151936890566</v>
+        <v>1.04844610560403</v>
       </c>
       <c r="C72" s="13" t="s">
         <v>140</v>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="B73" s="30" t="n">
         <f aca="false">'VPL e TIR'!B43</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C73" s="13" t="s">
         <v>142</v>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B74" s="30" t="n">
         <f aca="false">'VPL e TIR'!B44</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C74" s="13" t="s">
         <v>144</v>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B75" s="28" t="n">
         <f aca="false">AVERAGE('Projeção Mensal'!W18:W29)</f>
-        <v>2797.33416666667</v>
+        <v>3765.465</v>
       </c>
       <c r="C75" s="13" t="s">
         <v>146</v>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B79" s="15" t="n">
         <f aca="false">'Fluxo de Caixa'!$G$5+NPV((1+A79)^(1/12)-1,'Fluxo de Caixa'!$G$6:$G$29)</f>
-        <v>95036.919986325</v>
+        <v>138252.818253723</v>
       </c>
       <c r="C79" s="32" t="str">
         <f aca="false">IF(B79&gt;0,"Viável a esta taxa","Inviável a esta taxa")</f>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B80" s="15" t="n">
         <f aca="false">'Fluxo de Caixa'!$G$5+NPV((1+A80)^(1/12)-1,'Fluxo de Caixa'!$G$6:$G$29)</f>
-        <v>84862.163322548</v>
+        <v>126073.58365125</v>
       </c>
       <c r="C80" s="32" t="str">
         <f aca="false">IF(B80&gt;0,"Viável a esta taxa","Inviável a esta taxa")</f>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="B81" s="15" t="n">
         <f aca="false">'Fluxo de Caixa'!$G$5+NPV((1+A81)^(1/12)-1,'Fluxo de Caixa'!$G$6:$G$29)</f>
-        <v>77769.5508109088</v>
+        <v>117581.793796568</v>
       </c>
       <c r="C81" s="32" t="str">
         <f aca="false">IF(B81&gt;0,"Viável a esta taxa","Inviável a esta taxa")</f>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="B82" s="15" t="n">
         <f aca="false">'Fluxo de Caixa'!$G$5+NPV((1+A82)^(1/12)-1,'Fluxo de Caixa'!$G$6:$G$29)</f>
-        <v>73276.1226894992</v>
+        <v>112201.09352997</v>
       </c>
       <c r="C82" s="32" t="str">
         <f aca="false">IF(B82&gt;0,"Viável a esta taxa","Inviável a esta taxa")</f>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="B83" s="15" t="n">
         <f aca="false">'Fluxo de Caixa'!$G$5+NPV((1+A83)^(1/12)-1,'Fluxo de Caixa'!$G$6:$G$29)</f>
-        <v>64807.5818985632</v>
+        <v>102058.50248802</v>
       </c>
       <c r="C83" s="32" t="str">
         <f aca="false">IF(B83&gt;0,"Viável a esta taxa","Inviável a esta taxa")</f>
@@ -3502,11 +3502,11 @@
       </c>
       <c r="H11" s="15" t="n">
         <f aca="false">E11*'Premissas Precept'!$B$12</f>
-        <v>3166.16666666667</v>
+        <v>4999.5</v>
       </c>
       <c r="I11" s="22" t="n">
         <f aca="false">F11+G11+H11</f>
-        <v>32315.1666666667</v>
+        <v>34148.5</v>
       </c>
       <c r="J11" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I10)*12</f>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="L11" s="15" t="n">
         <f aca="false">I11*K11</f>
-        <v>5008.85083333333</v>
+        <v>5293.0175</v>
       </c>
       <c r="M11" s="15" t="n">
         <f aca="false">B11*'Premissas Precept'!$B$15</f>
@@ -3526,15 +3526,15 @@
       </c>
       <c r="N11" s="15" t="n">
         <f aca="false">I11*'Premissas Precept'!$B$16</f>
-        <v>646.303333333333</v>
+        <v>682.97</v>
       </c>
       <c r="O11" s="15" t="n">
         <f aca="false">(G11+H11)*'Premissas Precept'!$B$17</f>
-        <v>658.158333333333</v>
+        <v>749.825</v>
       </c>
       <c r="P11" s="15" t="n">
         <f aca="false">(G11+H11)*'Premissas Precept'!$B$18</f>
-        <v>4607.10833333333</v>
+        <v>5248.775</v>
       </c>
       <c r="Q11" s="15" t="n">
         <f aca="false">C11*'Premissas Precept'!$B$19+E11*'Premissas Precept'!$B$20</f>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="R11" s="22" t="n">
         <f aca="false">SUM(L11:Q11)</f>
-        <v>13160.4208333333</v>
+        <v>14214.5875</v>
       </c>
       <c r="S11" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -3550,19 +3550,19 @@
       </c>
       <c r="T11" s="15" t="n">
         <f aca="false">IF(A11&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I11,0)</f>
-        <v>6786.185</v>
+        <v>7171.185</v>
       </c>
       <c r="U11" s="22" t="n">
         <f aca="false">S11+T11</f>
-        <v>18786.185</v>
+        <v>19171.185</v>
       </c>
       <c r="V11" s="22" t="n">
         <f aca="false">I11-R11-U11</f>
-        <v>368.560833333333</v>
+        <v>762.727500000001</v>
       </c>
       <c r="W11" s="15" t="n">
         <f aca="false">T11/'Premissas Precept'!$B$45</f>
-        <v>969.455</v>
+        <v>1024.455</v>
       </c>
       <c r="X11" s="35" t="str">
         <f aca="false">IF(V11&gt;=0,"Sim","Não")</f>
@@ -3596,23 +3596,23 @@
       </c>
       <c r="H12" s="15" t="n">
         <f aca="false">E12*'Premissas Precept'!$B$12</f>
-        <v>3166.16666666667</v>
+        <v>4999.5</v>
       </c>
       <c r="I12" s="22" t="n">
         <f aca="false">F12+G12+H12</f>
-        <v>35906.1666666667</v>
+        <v>37739.5</v>
       </c>
       <c r="J12" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I11)*12</f>
-        <v>209954.333333333</v>
+        <v>213621</v>
       </c>
       <c r="K12" s="38" t="n">
         <f aca="false">IF(J12&lt;=0,'Premissas Precept'!$C$24,(J12*LOOKUP(J12,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J12,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J12)</f>
-        <v>0.158566767693927</v>
+        <v>0.158934655300743</v>
       </c>
       <c r="L12" s="15" t="n">
         <f aca="false">I12*K12</f>
-        <v>5693.52478861276</v>
+        <v>5998.11442372239</v>
       </c>
       <c r="M12" s="15" t="n">
         <f aca="false">B12*'Premissas Precept'!$B$15</f>
@@ -3620,15 +3620,15 @@
       </c>
       <c r="N12" s="15" t="n">
         <f aca="false">I12*'Premissas Precept'!$B$16</f>
-        <v>718.123333333333</v>
+        <v>754.79</v>
       </c>
       <c r="O12" s="15" t="n">
         <f aca="false">(G12+H12)*'Premissas Precept'!$B$17</f>
-        <v>658.158333333333</v>
+        <v>749.825</v>
       </c>
       <c r="P12" s="15" t="n">
         <f aca="false">(G12+H12)*'Premissas Precept'!$B$18</f>
-        <v>4607.10833333333</v>
+        <v>5248.775</v>
       </c>
       <c r="Q12" s="15" t="n">
         <f aca="false">C12*'Premissas Precept'!$B$19+E12*'Premissas Precept'!$B$20</f>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="R12" s="22" t="n">
         <f aca="false">SUM(L12:Q12)</f>
-        <v>14186.9147886128</v>
+        <v>15261.5044237224</v>
       </c>
       <c r="S12" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -3644,19 +3644,19 @@
       </c>
       <c r="T12" s="15" t="n">
         <f aca="false">IF(A12&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I12,0)</f>
-        <v>7540.295</v>
+        <v>7925.295</v>
       </c>
       <c r="U12" s="22" t="n">
         <f aca="false">S12+T12</f>
-        <v>19540.295</v>
+        <v>19925.295</v>
       </c>
       <c r="V12" s="22" t="n">
         <f aca="false">I12-R12-U12</f>
-        <v>2178.95687805391</v>
+        <v>2552.70057627762</v>
       </c>
       <c r="W12" s="15" t="n">
         <f aca="false">T12/'Premissas Precept'!$B$45</f>
-        <v>1077.185</v>
+        <v>1132.185</v>
       </c>
       <c r="X12" s="35" t="str">
         <f aca="false">IF(V12&gt;=0,"Sim","Não")</f>
@@ -3690,23 +3690,23 @@
       </c>
       <c r="H13" s="15" t="n">
         <f aca="false">E13*'Premissas Precept'!$B$12</f>
-        <v>6332.33333333333</v>
+        <v>9999</v>
       </c>
       <c r="I13" s="22" t="n">
         <f aca="false">F13+G13+H13</f>
-        <v>41466.3333333333</v>
+        <v>45133</v>
       </c>
       <c r="J13" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I12)*12</f>
-        <v>241514.285714286</v>
+        <v>247800</v>
       </c>
       <c r="K13" s="38" t="n">
         <f aca="false">IF(J13&lt;=0,'Premissas Precept'!$C$24,(J13*LOOKUP(J13,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J13,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J13)</f>
-        <v>0.161367561812374</v>
+        <v>0.1618401937046</v>
       </c>
       <c r="L13" s="15" t="n">
         <f aca="false">I13*K13</f>
-        <v>6691.32110729919</v>
+        <v>7304.33346246973</v>
       </c>
       <c r="M13" s="15" t="n">
         <f aca="false">B13*'Premissas Precept'!$B$15</f>
@@ -3714,15 +3714,15 @@
       </c>
       <c r="N13" s="15" t="n">
         <f aca="false">I13*'Premissas Precept'!$B$16</f>
-        <v>829.326666666667</v>
+        <v>902.66</v>
       </c>
       <c r="O13" s="15" t="n">
         <f aca="false">(G13+H13)*'Premissas Precept'!$B$17</f>
-        <v>816.466666666667</v>
+        <v>999.8</v>
       </c>
       <c r="P13" s="15" t="n">
         <f aca="false">(G13+H13)*'Premissas Precept'!$B$18</f>
-        <v>5715.26666666667</v>
+        <v>6998.6</v>
       </c>
       <c r="Q13" s="15" t="n">
         <f aca="false">C13*'Premissas Precept'!$B$19+E13*'Premissas Precept'!$B$20</f>
@@ -3730,7 +3730,7 @@
       </c>
       <c r="R13" s="22" t="n">
         <f aca="false">SUM(L13:Q13)</f>
-        <v>16942.3811072992</v>
+        <v>19095.3934624697</v>
       </c>
       <c r="S13" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -3738,19 +3738,19 @@
       </c>
       <c r="T13" s="15" t="n">
         <f aca="false">IF(A13&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I13,0)</f>
-        <v>8707.93</v>
+        <v>9477.93</v>
       </c>
       <c r="U13" s="22" t="n">
         <f aca="false">S13+T13</f>
-        <v>20707.93</v>
+        <v>21477.93</v>
       </c>
       <c r="V13" s="22" t="n">
         <f aca="false">I13-R13-U13</f>
-        <v>3816.02222603415</v>
+        <v>4559.67653753027</v>
       </c>
       <c r="W13" s="15" t="n">
         <f aca="false">T13/'Premissas Precept'!$B$45</f>
-        <v>1243.99</v>
+        <v>1353.99</v>
       </c>
       <c r="X13" s="35" t="str">
         <f aca="false">IF(V13&gt;=0,"Sim","Não")</f>
@@ -3784,23 +3784,23 @@
       </c>
       <c r="H14" s="15" t="n">
         <f aca="false">E14*'Premissas Precept'!$B$12</f>
-        <v>6332.33333333333</v>
+        <v>9999</v>
       </c>
       <c r="I14" s="22" t="n">
         <f aca="false">F14+G14+H14</f>
-        <v>55054.3333333333</v>
+        <v>58721</v>
       </c>
       <c r="J14" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I13)*12</f>
-        <v>273524.5</v>
+        <v>284524.5</v>
       </c>
       <c r="K14" s="38" t="n">
         <f aca="false">IF(J14&lt;=0,'Premissas Precept'!$C$24,(J14*LOOKUP(J14,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J14,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J14)</f>
-        <v>0.163548091670033</v>
+        <v>0.164184138799998</v>
       </c>
       <c r="L14" s="15" t="n">
         <f aca="false">I14*K14</f>
-        <v>9004.03115483256</v>
+        <v>9641.05681447468</v>
       </c>
       <c r="M14" s="15" t="n">
         <f aca="false">B14*'Premissas Precept'!$B$15</f>
@@ -3808,15 +3808,15 @@
       </c>
       <c r="N14" s="15" t="n">
         <f aca="false">I14*'Premissas Precept'!$B$16</f>
-        <v>1101.08666666667</v>
+        <v>1174.42</v>
       </c>
       <c r="O14" s="15" t="n">
         <f aca="false">(G14+H14)*'Premissas Precept'!$B$17</f>
-        <v>1316.31666666667</v>
+        <v>1499.65</v>
       </c>
       <c r="P14" s="15" t="n">
         <f aca="false">(G14+H14)*'Premissas Precept'!$B$18</f>
-        <v>9214.21666666667</v>
+        <v>10497.55</v>
       </c>
       <c r="Q14" s="15" t="n">
         <f aca="false">C14*'Premissas Precept'!$B$19+E14*'Premissas Precept'!$B$20</f>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="R14" s="22" t="n">
         <f aca="false">SUM(L14:Q14)</f>
-        <v>24395.6511548326</v>
+        <v>26572.6768144747</v>
       </c>
       <c r="S14" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -3832,19 +3832,19 @@
       </c>
       <c r="T14" s="15" t="n">
         <f aca="false">IF(A14&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I14,0)</f>
-        <v>11561.41</v>
+        <v>12331.41</v>
       </c>
       <c r="U14" s="22" t="n">
         <f aca="false">S14+T14</f>
-        <v>23561.41</v>
+        <v>24331.41</v>
       </c>
       <c r="V14" s="22" t="n">
         <f aca="false">I14-R14-U14</f>
-        <v>7097.27217850077</v>
+        <v>7816.91318552533</v>
       </c>
       <c r="W14" s="15" t="n">
         <f aca="false">T14/'Premissas Precept'!$B$45</f>
-        <v>1651.63</v>
+        <v>1761.63</v>
       </c>
       <c r="X14" s="35" t="str">
         <f aca="false">IF(V14&gt;=0,"Sim","Não")</f>
@@ -3878,23 +3878,23 @@
       </c>
       <c r="H15" s="15" t="n">
         <f aca="false">E15*'Premissas Precept'!$B$12</f>
-        <v>9498.5</v>
+        <v>14998.5</v>
       </c>
       <c r="I15" s="22" t="n">
         <f aca="false">F15+G15+H15</f>
-        <v>50617.5</v>
+        <v>56117.5</v>
       </c>
       <c r="J15" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I14)*12</f>
-        <v>316538.666666667</v>
+        <v>331205.333333333</v>
       </c>
       <c r="K15" s="38" t="n">
         <f aca="false">IF(J15&lt;=0,'Premissas Precept'!$C$24,(J15*LOOKUP(J15,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J15,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J15)</f>
-        <v>0.165783727317147</v>
+        <v>0.166413262266308</v>
       </c>
       <c r="L15" s="15" t="n">
         <f aca="false">I15*K15</f>
-        <v>8391.5578174757</v>
+        <v>9338.69624522955</v>
       </c>
       <c r="M15" s="15" t="n">
         <f aca="false">B15*'Premissas Precept'!$B$15</f>
@@ -3902,15 +3902,15 @@
       </c>
       <c r="N15" s="15" t="n">
         <f aca="false">I15*'Premissas Precept'!$B$16</f>
-        <v>1012.35</v>
+        <v>1122.35</v>
       </c>
       <c r="O15" s="15" t="n">
         <f aca="false">(G15+H15)*'Premissas Precept'!$B$17</f>
-        <v>974.775</v>
+        <v>1249.775</v>
       </c>
       <c r="P15" s="15" t="n">
         <f aca="false">(G15+H15)*'Premissas Precept'!$B$18</f>
-        <v>6823.425</v>
+        <v>8748.425</v>
       </c>
       <c r="Q15" s="15" t="n">
         <f aca="false">C15*'Premissas Precept'!$B$19+E15*'Premissas Precept'!$B$20</f>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="R15" s="22" t="n">
         <f aca="false">SUM(L15:Q15)</f>
-        <v>20742.1078174757</v>
+        <v>23999.2462452295</v>
       </c>
       <c r="S15" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -3926,19 +3926,19 @@
       </c>
       <c r="T15" s="15" t="n">
         <f aca="false">IF(A15&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I15,0)</f>
-        <v>10629.675</v>
+        <v>11784.675</v>
       </c>
       <c r="U15" s="22" t="n">
         <f aca="false">S15+T15</f>
-        <v>22629.675</v>
+        <v>23784.675</v>
       </c>
       <c r="V15" s="22" t="n">
         <f aca="false">I15-R15-U15</f>
-        <v>7245.71718252431</v>
+        <v>8333.57875477045</v>
       </c>
       <c r="W15" s="15" t="n">
         <f aca="false">T15/'Premissas Precept'!$B$45</f>
-        <v>1518.525</v>
+        <v>1683.525</v>
       </c>
       <c r="X15" s="35" t="str">
         <f aca="false">IF(V15&gt;=0,"Sim","Não")</f>
@@ -3972,23 +3972,23 @@
       </c>
       <c r="H16" s="15" t="n">
         <f aca="false">E16*'Premissas Precept'!$B$12</f>
-        <v>9498.5</v>
+        <v>14998.5</v>
       </c>
       <c r="I16" s="22" t="n">
         <f aca="false">F16+G16+H16</f>
-        <v>64205.5</v>
+        <v>69705.5</v>
       </c>
       <c r="J16" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I15)*12</f>
-        <v>345625.8</v>
+        <v>365425.8</v>
       </c>
       <c r="K16" s="38" t="n">
         <f aca="false">IF(J16&lt;=0,'Premissas Precept'!$C$24,(J16*LOOKUP(J16,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J16,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J16)</f>
-        <v>0.166980138635484</v>
+        <v>0.167908316818353</v>
       </c>
       <c r="L16" s="15" t="n">
         <f aca="false">I16*K16</f>
-        <v>10721.0432911606</v>
+        <v>11704.1331779817</v>
       </c>
       <c r="M16" s="15" t="n">
         <f aca="false">B16*'Premissas Precept'!$B$15</f>
@@ -3996,15 +3996,15 @@
       </c>
       <c r="N16" s="15" t="n">
         <f aca="false">I16*'Premissas Precept'!$B$16</f>
-        <v>1284.11</v>
+        <v>1394.11</v>
       </c>
       <c r="O16" s="15" t="n">
         <f aca="false">(G16+H16)*'Premissas Precept'!$B$17</f>
-        <v>1474.625</v>
+        <v>1749.625</v>
       </c>
       <c r="P16" s="15" t="n">
         <f aca="false">(G16+H16)*'Premissas Precept'!$B$18</f>
-        <v>10322.375</v>
+        <v>12247.375</v>
       </c>
       <c r="Q16" s="15" t="n">
         <f aca="false">C16*'Premissas Precept'!$B$19+E16*'Premissas Precept'!$B$20</f>
@@ -4012,7 +4012,7 @@
       </c>
       <c r="R16" s="22" t="n">
         <f aca="false">SUM(L16:Q16)</f>
-        <v>28212.1532911606</v>
+        <v>31505.2431779817</v>
       </c>
       <c r="S16" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4020,19 +4020,19 @@
       </c>
       <c r="T16" s="15" t="n">
         <f aca="false">IF(A16&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I16,0)</f>
-        <v>13483.155</v>
+        <v>14638.155</v>
       </c>
       <c r="U16" s="22" t="n">
         <f aca="false">S16+T16</f>
-        <v>25483.155</v>
+        <v>26638.155</v>
       </c>
       <c r="V16" s="22" t="n">
         <f aca="false">I16-R16-U16</f>
-        <v>10510.1917088394</v>
+        <v>11562.1018220183</v>
       </c>
       <c r="W16" s="15" t="n">
         <f aca="false">T16/'Premissas Precept'!$B$45</f>
-        <v>1926.165</v>
+        <v>2091.165</v>
       </c>
       <c r="X16" s="35" t="str">
         <f aca="false">IF(V16&gt;=0,"Sim","Não")</f>
@@ -4066,23 +4066,23 @@
       </c>
       <c r="H17" s="15" t="n">
         <f aca="false">E17*'Premissas Precept'!$B$12</f>
-        <v>9498.5</v>
+        <v>14998.5</v>
       </c>
       <c r="I17" s="22" t="n">
         <f aca="false">F17+G17+H17</f>
-        <v>56602.5</v>
+        <v>62102.5</v>
       </c>
       <c r="J17" s="15" t="n">
         <f aca="false">AVERAGE(I$6:I16)*12</f>
-        <v>384247.636363636</v>
+        <v>408247.636363636</v>
       </c>
       <c r="K17" s="38" t="n">
         <f aca="false">IF(J17&lt;=0,'Premissas Precept'!$C$24,(J17*LOOKUP(J17,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J17,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J17)</f>
-        <v>0.169235365261607</v>
+        <v>0.170750012692831</v>
       </c>
       <c r="L17" s="15" t="n">
         <f aca="false">I17*K17</f>
-        <v>9579.1447622201</v>
+        <v>10604.0026632565</v>
       </c>
       <c r="M17" s="15" t="n">
         <f aca="false">B17*'Premissas Precept'!$B$15</f>
@@ -4090,15 +4090,15 @@
       </c>
       <c r="N17" s="15" t="n">
         <f aca="false">I17*'Premissas Precept'!$B$16</f>
-        <v>1132.05</v>
+        <v>1242.05</v>
       </c>
       <c r="O17" s="15" t="n">
         <f aca="false">(G17+H17)*'Premissas Precept'!$B$17</f>
-        <v>974.775</v>
+        <v>1249.775</v>
       </c>
       <c r="P17" s="15" t="n">
         <f aca="false">(G17+H17)*'Premissas Precept'!$B$18</f>
-        <v>6823.425</v>
+        <v>8748.425</v>
       </c>
       <c r="Q17" s="15" t="n">
         <f aca="false">C17*'Premissas Precept'!$B$19+E17*'Premissas Precept'!$B$20</f>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="R17" s="22" t="n">
         <f aca="false">SUM(L17:Q17)</f>
-        <v>22499.3947622201</v>
+        <v>25834.2526632565</v>
       </c>
       <c r="S17" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4114,19 +4114,19 @@
       </c>
       <c r="T17" s="15" t="n">
         <f aca="false">IF(A17&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I17,0)</f>
-        <v>11886.525</v>
+        <v>13041.525</v>
       </c>
       <c r="U17" s="22" t="n">
         <f aca="false">S17+T17</f>
-        <v>23886.525</v>
+        <v>25041.525</v>
       </c>
       <c r="V17" s="22" t="n">
         <f aca="false">I17-R17-U17</f>
-        <v>10216.5802377799</v>
+        <v>11226.7223367435</v>
       </c>
       <c r="W17" s="15" t="n">
         <f aca="false">T17/'Premissas Precept'!$B$45</f>
-        <v>1698.075</v>
+        <v>1863.075</v>
       </c>
       <c r="X17" s="35" t="str">
         <f aca="false">IF(V17&gt;=0,"Sim","Não")</f>
@@ -4141,7 +4141,7 @@
         <v>34</v>
       </c>
       <c r="C18" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" s="36" t="n">
         <v>1</v>
@@ -4156,27 +4156,27 @@
       </c>
       <c r="G18" s="15" t="n">
         <f aca="false">C18*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>39988</v>
       </c>
       <c r="H18" s="15" t="n">
         <f aca="false">E18*'Premissas Precept'!$B$12</f>
-        <v>12664.6666666667</v>
+        <v>19998</v>
       </c>
       <c r="I18" s="22" t="n">
         <f aca="false">F18+G18+H18</f>
-        <v>73356.6666666667</v>
+        <v>100684</v>
       </c>
       <c r="J18" s="15" t="n">
         <f aca="false">SUM(I6:I17)</f>
-        <v>408829.5</v>
+        <v>436329.5</v>
       </c>
       <c r="K18" s="38" t="n">
         <f aca="false">IF(J18&lt;=0,'Premissas Precept'!$C$24,(J18*LOOKUP(J18,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J18,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J18)</f>
-        <v>0.170784526312314</v>
+        <v>0.172310725036927</v>
       </c>
       <c r="L18" s="15" t="n">
         <f aca="false">I18*K18</f>
-        <v>12528.183568517</v>
+        <v>17348.933039618</v>
       </c>
       <c r="M18" s="15" t="n">
         <f aca="false">B18*'Premissas Precept'!$B$15</f>
@@ -4184,23 +4184,23 @@
       </c>
       <c r="N18" s="15" t="n">
         <f aca="false">I18*'Premissas Precept'!$B$16</f>
-        <v>1467.13333333333</v>
+        <v>2013.68</v>
       </c>
       <c r="O18" s="15" t="n">
         <f aca="false">(G18+H18)*'Premissas Precept'!$B$17</f>
-        <v>1632.93333333333</v>
+        <v>2999.3</v>
       </c>
       <c r="P18" s="15" t="n">
         <f aca="false">(G18+H18)*'Premissas Precept'!$B$18</f>
-        <v>11430.5333333333</v>
+        <v>20995.1</v>
       </c>
       <c r="Q18" s="15" t="n">
         <f aca="false">C18*'Premissas Precept'!$B$19+E18*'Premissas Precept'!$B$20</f>
-        <v>2000</v>
+        <v>3200</v>
       </c>
       <c r="R18" s="22" t="n">
         <f aca="false">SUM(L18:Q18)</f>
-        <v>32118.783568517</v>
+        <v>49617.013039618</v>
       </c>
       <c r="S18" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4208,19 +4208,19 @@
       </c>
       <c r="T18" s="15" t="n">
         <f aca="false">IF(A18&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I18,0)</f>
-        <v>15404.9</v>
+        <v>21143.64</v>
       </c>
       <c r="U18" s="22" t="n">
         <f aca="false">S18+T18</f>
-        <v>27404.9</v>
+        <v>33143.64</v>
       </c>
       <c r="V18" s="22" t="n">
         <f aca="false">I18-R18-U18</f>
-        <v>13832.9830981497</v>
+        <v>17923.346960382</v>
       </c>
       <c r="W18" s="15" t="n">
         <f aca="false">T18/'Premissas Precept'!$B$45</f>
-        <v>2200.7</v>
+        <v>3020.52</v>
       </c>
       <c r="X18" s="35" t="str">
         <f aca="false">IF(V18&gt;=0,"Sim","Não")</f>
@@ -4235,7 +4235,7 @@
         <v>36</v>
       </c>
       <c r="C19" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" s="36" t="n">
         <v>1</v>
@@ -4250,27 +4250,27 @@
       </c>
       <c r="G19" s="15" t="n">
         <f aca="false">C19*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>39988</v>
       </c>
       <c r="H19" s="15" t="n">
         <f aca="false">E19*'Premissas Precept'!$B$12</f>
-        <v>12664.6666666667</v>
+        <v>19998</v>
       </c>
       <c r="I19" s="22" t="n">
         <f aca="false">F19+G19+H19</f>
-        <v>75750.6666666667</v>
+        <v>103078</v>
       </c>
       <c r="J19" s="15" t="n">
         <f aca="false">SUM(I7:I18)</f>
-        <v>477398.166666667</v>
+        <v>532225.5</v>
       </c>
       <c r="K19" s="38" t="n">
         <f aca="false">IF(J19&lt;=0,'Premissas Precept'!$C$24,(J19*LOOKUP(J19,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J19,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J19)</f>
-        <v>0.174262593174321</v>
+        <v>0.176398861948554</v>
       </c>
       <c r="L19" s="15" t="n">
         <f aca="false">I19*K19</f>
-        <v>13200.5076080169</v>
+        <v>18182.841891933</v>
       </c>
       <c r="M19" s="15" t="n">
         <f aca="false">B19*'Premissas Precept'!$B$15</f>
@@ -4278,23 +4278,23 @@
       </c>
       <c r="N19" s="15" t="n">
         <f aca="false">I19*'Premissas Precept'!$B$16</f>
-        <v>1515.01333333333</v>
+        <v>2061.56</v>
       </c>
       <c r="O19" s="15" t="n">
         <f aca="false">(G19+H19)*'Premissas Precept'!$B$17</f>
-        <v>1632.93333333333</v>
+        <v>2999.3</v>
       </c>
       <c r="P19" s="15" t="n">
         <f aca="false">(G19+H19)*'Premissas Precept'!$B$18</f>
-        <v>11430.5333333333</v>
+        <v>20995.1</v>
       </c>
       <c r="Q19" s="15" t="n">
         <f aca="false">C19*'Premissas Precept'!$B$19+E19*'Premissas Precept'!$B$20</f>
-        <v>2000</v>
+        <v>3200</v>
       </c>
       <c r="R19" s="22" t="n">
         <f aca="false">SUM(L19:Q19)</f>
-        <v>33018.9876080169</v>
+        <v>50678.801891933</v>
       </c>
       <c r="S19" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4302,19 +4302,19 @@
       </c>
       <c r="T19" s="15" t="n">
         <f aca="false">IF(A19&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I19,0)</f>
-        <v>15907.64</v>
+        <v>21646.38</v>
       </c>
       <c r="U19" s="22" t="n">
         <f aca="false">S19+T19</f>
-        <v>27907.64</v>
+        <v>33646.38</v>
       </c>
       <c r="V19" s="22" t="n">
         <f aca="false">I19-R19-U19</f>
-        <v>14824.0390586497</v>
+        <v>18752.818108067</v>
       </c>
       <c r="W19" s="15" t="n">
         <f aca="false">T19/'Premissas Precept'!$B$45</f>
-        <v>2272.52</v>
+        <v>3092.34</v>
       </c>
       <c r="X19" s="35" t="str">
         <f aca="false">IF(V19&gt;=0,"Sim","Não")</f>
@@ -4329,7 +4329,7 @@
         <v>38</v>
       </c>
       <c r="C20" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" s="36" t="n">
         <v>1</v>
@@ -4344,27 +4344,27 @@
       </c>
       <c r="G20" s="15" t="n">
         <f aca="false">C20*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>39988</v>
       </c>
       <c r="H20" s="15" t="n">
         <f aca="false">E20*'Premissas Precept'!$B$12</f>
-        <v>15830.8333333333</v>
+        <v>24997.5</v>
       </c>
       <c r="I20" s="22" t="n">
         <f aca="false">F20+G20+H20</f>
-        <v>81310.8333333333</v>
+        <v>110471.5</v>
       </c>
       <c r="J20" s="15" t="n">
         <f aca="false">SUM(I8:I19)</f>
-        <v>545966.833333333</v>
+        <v>628121.5</v>
       </c>
       <c r="K20" s="38" t="n">
         <f aca="false">IF(J20&lt;=0,'Premissas Precept'!$C$24,(J20*LOOKUP(J20,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J20,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J20)</f>
-        <v>0.176867030384324</v>
+        <v>0.179238718146091</v>
       </c>
       <c r="L20" s="15" t="n">
         <f aca="false">I20*K20</f>
-        <v>14381.2056297414</v>
+        <v>19800.7700516759</v>
       </c>
       <c r="M20" s="15" t="n">
         <f aca="false">B20*'Premissas Precept'!$B$15</f>
@@ -4372,23 +4372,23 @@
       </c>
       <c r="N20" s="15" t="n">
         <f aca="false">I20*'Premissas Precept'!$B$16</f>
-        <v>1626.21666666667</v>
+        <v>2209.43</v>
       </c>
       <c r="O20" s="15" t="n">
         <f aca="false">(G20+H20)*'Premissas Precept'!$B$17</f>
-        <v>1791.24166666667</v>
+        <v>3249.275</v>
       </c>
       <c r="P20" s="15" t="n">
         <f aca="false">(G20+H20)*'Premissas Precept'!$B$18</f>
-        <v>12538.6916666667</v>
+        <v>22744.925</v>
       </c>
       <c r="Q20" s="15" t="n">
         <f aca="false">C20*'Premissas Precept'!$B$19+E20*'Premissas Precept'!$B$20</f>
-        <v>2200</v>
+        <v>3400</v>
       </c>
       <c r="R20" s="22" t="n">
         <f aca="false">SUM(L20:Q20)</f>
-        <v>35957.3556297414</v>
+        <v>54824.4000516759</v>
       </c>
       <c r="S20" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4396,19 +4396,19 @@
       </c>
       <c r="T20" s="15" t="n">
         <f aca="false">IF(A20&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I20,0)</f>
-        <v>17075.275</v>
+        <v>23199.015</v>
       </c>
       <c r="U20" s="22" t="n">
         <f aca="false">S20+T20</f>
-        <v>29075.275</v>
+        <v>35199.015</v>
       </c>
       <c r="V20" s="22" t="n">
         <f aca="false">I20-R20-U20</f>
-        <v>16278.2027035919</v>
+        <v>20448.0849483241</v>
       </c>
       <c r="W20" s="15" t="n">
         <f aca="false">T20/'Premissas Precept'!$B$45</f>
-        <v>2439.325</v>
+        <v>3314.145</v>
       </c>
       <c r="X20" s="35" t="str">
         <f aca="false">IF(V20&gt;=0,"Sim","Não")</f>
@@ -4423,7 +4423,7 @@
         <v>40</v>
       </c>
       <c r="C21" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" s="36" t="n">
         <v>1</v>
@@ -4438,27 +4438,27 @@
       </c>
       <c r="G21" s="15" t="n">
         <f aca="false">C21*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>39988</v>
       </c>
       <c r="H21" s="15" t="n">
         <f aca="false">E21*'Premissas Precept'!$B$12</f>
-        <v>15830.8333333333</v>
+        <v>24997.5</v>
       </c>
       <c r="I21" s="22" t="n">
         <f aca="false">F21+G21+H21</f>
-        <v>83704.8333333333</v>
+        <v>112865.5</v>
       </c>
       <c r="J21" s="15" t="n">
         <f aca="false">SUM(I9:I20)</f>
-        <v>616504.666666667</v>
+        <v>727820</v>
       </c>
       <c r="K21" s="38" t="n">
         <f aca="false">IF(J21&lt;=0,'Premissas Precept'!$C$24,(J21*LOOKUP(J21,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J21,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J21)</f>
-        <v>0.178941727394332</v>
+        <v>0.181505179852161</v>
       </c>
       <c r="L21" s="15" t="n">
         <f aca="false">I21*K21</f>
-        <v>14978.2874679213</v>
+        <v>20485.6728766041</v>
       </c>
       <c r="M21" s="15" t="n">
         <f aca="false">B21*'Premissas Precept'!$B$15</f>
@@ -4466,23 +4466,23 @@
       </c>
       <c r="N21" s="15" t="n">
         <f aca="false">I21*'Premissas Precept'!$B$16</f>
-        <v>1674.09666666667</v>
+        <v>2257.31</v>
       </c>
       <c r="O21" s="15" t="n">
         <f aca="false">(G21+H21)*'Premissas Precept'!$B$17</f>
-        <v>1791.24166666667</v>
+        <v>3249.275</v>
       </c>
       <c r="P21" s="15" t="n">
         <f aca="false">(G21+H21)*'Premissas Precept'!$B$18</f>
-        <v>12538.6916666667</v>
+        <v>22744.925</v>
       </c>
       <c r="Q21" s="15" t="n">
         <f aca="false">C21*'Premissas Precept'!$B$19+E21*'Premissas Precept'!$B$20</f>
-        <v>2200</v>
+        <v>3400</v>
       </c>
       <c r="R21" s="22" t="n">
         <f aca="false">SUM(L21:Q21)</f>
-        <v>36782.3174679213</v>
+        <v>55737.1828766041</v>
       </c>
       <c r="S21" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4490,19 +4490,19 @@
       </c>
       <c r="T21" s="15" t="n">
         <f aca="false">IF(A21&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I21,0)</f>
-        <v>17578.015</v>
+        <v>23701.755</v>
       </c>
       <c r="U21" s="22" t="n">
         <f aca="false">S21+T21</f>
-        <v>29578.015</v>
+        <v>35701.755</v>
       </c>
       <c r="V21" s="22" t="n">
         <f aca="false">I21-R21-U21</f>
-        <v>17344.500865412</v>
+        <v>21426.5621233959</v>
       </c>
       <c r="W21" s="15" t="n">
         <f aca="false">T21/'Premissas Precept'!$B$45</f>
-        <v>2511.145</v>
+        <v>3385.965</v>
       </c>
       <c r="X21" s="35" t="str">
         <f aca="false">IF(V21&gt;=0,"Sim","Não")</f>
@@ -4517,7 +4517,7 @@
         <v>42</v>
       </c>
       <c r="C22" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D22" s="36" t="n">
         <v>1</v>
@@ -4532,27 +4532,27 @@
       </c>
       <c r="G22" s="15" t="n">
         <f aca="false">C22*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>39988</v>
       </c>
       <c r="H22" s="15" t="n">
         <f aca="false">E22*'Premissas Precept'!$B$12</f>
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="I22" s="22" t="n">
         <f aca="false">F22+G22+H22</f>
-        <v>89265</v>
+        <v>120259</v>
       </c>
       <c r="J22" s="15" t="n">
         <f aca="false">SUM(I10:I21)</f>
-        <v>677045.5</v>
+        <v>817521.5</v>
       </c>
       <c r="K22" s="38" t="n">
         <f aca="false">IF(J22&lt;=0,'Premissas Precept'!$C$24,(J22*LOOKUP(J22,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J22,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J22)</f>
-        <v>0.180377644486227</v>
+        <v>0.184083118914915</v>
       </c>
       <c r="L22" s="15" t="n">
         <f aca="false">I22*K22</f>
-        <v>16101.4104350631</v>
+        <v>22137.6517975888</v>
       </c>
       <c r="M22" s="15" t="n">
         <f aca="false">B22*'Premissas Precept'!$B$15</f>
@@ -4560,23 +4560,23 @@
       </c>
       <c r="N22" s="15" t="n">
         <f aca="false">I22*'Premissas Precept'!$B$16</f>
-        <v>1785.3</v>
+        <v>2405.18</v>
       </c>
       <c r="O22" s="15" t="n">
         <f aca="false">(G22+H22)*'Premissas Precept'!$B$17</f>
-        <v>1949.55</v>
+        <v>3499.25</v>
       </c>
       <c r="P22" s="15" t="n">
         <f aca="false">(G22+H22)*'Premissas Precept'!$B$18</f>
-        <v>13646.85</v>
+        <v>24494.75</v>
       </c>
       <c r="Q22" s="15" t="n">
         <f aca="false">C22*'Premissas Precept'!$B$19+E22*'Premissas Precept'!$B$20</f>
-        <v>2400</v>
+        <v>3600</v>
       </c>
       <c r="R22" s="22" t="n">
         <f aca="false">SUM(L22:Q22)</f>
-        <v>39663.1104350631</v>
+        <v>59916.8317975888</v>
       </c>
       <c r="S22" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4584,19 +4584,19 @@
       </c>
       <c r="T22" s="15" t="n">
         <f aca="false">IF(A22&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I22,0)</f>
-        <v>18745.65</v>
+        <v>25254.39</v>
       </c>
       <c r="U22" s="22" t="n">
         <f aca="false">S22+T22</f>
-        <v>30745.65</v>
+        <v>37254.39</v>
       </c>
       <c r="V22" s="22" t="n">
         <f aca="false">I22-R22-U22</f>
-        <v>18856.2395649369</v>
+        <v>23087.7782024112</v>
       </c>
       <c r="W22" s="15" t="n">
         <f aca="false">T22/'Premissas Precept'!$B$45</f>
-        <v>2677.95</v>
+        <v>3607.77</v>
       </c>
       <c r="X22" s="35" t="str">
         <f aca="false">IF(V22&gt;=0,"Sim","Não")</f>
@@ -4611,7 +4611,7 @@
         <v>44</v>
       </c>
       <c r="C23" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D23" s="36" t="n">
         <v>1</v>
@@ -4626,27 +4626,27 @@
       </c>
       <c r="G23" s="15" t="n">
         <f aca="false">C23*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>39988</v>
       </c>
       <c r="H23" s="15" t="n">
         <f aca="false">E23*'Premissas Precept'!$B$12</f>
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="I23" s="22" t="n">
         <f aca="false">F23+G23+H23</f>
-        <v>91659</v>
+        <v>122653</v>
       </c>
       <c r="J23" s="15" t="n">
         <f aca="false">SUM(I11:I22)</f>
-        <v>739555.5</v>
+        <v>911025.5</v>
       </c>
       <c r="K23" s="38" t="n">
         <f aca="false">IF(J23&lt;=0,'Premissas Precept'!$C$24,(J23*LOOKUP(J23,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J23,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J23)</f>
-        <v>0.181878003070763</v>
+        <v>0.186229943618483</v>
       </c>
       <c r="L23" s="15" t="n">
         <f aca="false">I23*K23</f>
-        <v>16670.7558834631</v>
+        <v>22841.6612746378</v>
       </c>
       <c r="M23" s="15" t="n">
         <f aca="false">B23*'Premissas Precept'!$B$15</f>
@@ -4654,23 +4654,23 @@
       </c>
       <c r="N23" s="15" t="n">
         <f aca="false">I23*'Premissas Precept'!$B$16</f>
-        <v>1833.18</v>
+        <v>2453.06</v>
       </c>
       <c r="O23" s="15" t="n">
         <f aca="false">(G23+H23)*'Premissas Precept'!$B$17</f>
-        <v>1949.55</v>
+        <v>3499.25</v>
       </c>
       <c r="P23" s="15" t="n">
         <f aca="false">(G23+H23)*'Premissas Precept'!$B$18</f>
-        <v>13646.85</v>
+        <v>24494.75</v>
       </c>
       <c r="Q23" s="15" t="n">
         <f aca="false">C23*'Premissas Precept'!$B$19+E23*'Premissas Precept'!$B$20</f>
-        <v>2400</v>
+        <v>3600</v>
       </c>
       <c r="R23" s="22" t="n">
         <f aca="false">SUM(L23:Q23)</f>
-        <v>40460.3358834631</v>
+        <v>60848.7212746378</v>
       </c>
       <c r="S23" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4678,19 +4678,19 @@
       </c>
       <c r="T23" s="15" t="n">
         <f aca="false">IF(A23&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I23,0)</f>
-        <v>19248.39</v>
+        <v>25757.13</v>
       </c>
       <c r="U23" s="22" t="n">
         <f aca="false">S23+T23</f>
-        <v>31248.39</v>
+        <v>37757.13</v>
       </c>
       <c r="V23" s="22" t="n">
         <f aca="false">I23-R23-U23</f>
-        <v>19950.2741165369</v>
+        <v>24047.1487253622</v>
       </c>
       <c r="W23" s="15" t="n">
         <f aca="false">T23/'Premissas Precept'!$B$45</f>
-        <v>2749.77</v>
+        <v>3679.59</v>
       </c>
       <c r="X23" s="35" t="str">
         <f aca="false">IF(V23&gt;=0,"Sim","Não")</f>
@@ -4705,7 +4705,7 @@
         <v>46</v>
       </c>
       <c r="C24" s="36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D24" s="36" t="n">
         <v>1</v>
@@ -4720,27 +4720,27 @@
       </c>
       <c r="G24" s="15" t="n">
         <f aca="false">C24*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>49985</v>
       </c>
       <c r="H24" s="15" t="n">
         <f aca="false">E24*'Premissas Precept'!$B$12</f>
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="I24" s="22" t="n">
         <f aca="false">F24+G24+H24</f>
-        <v>94053</v>
+        <v>135044</v>
       </c>
       <c r="J24" s="15" t="n">
         <f aca="false">SUM(I12:I23)</f>
-        <v>798899.333333333</v>
+        <v>999530</v>
       </c>
       <c r="K24" s="38" t="n">
         <f aca="false">IF(J24&lt;=0,'Premissas Precept'!$C$24,(J24*LOOKUP(J24,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J24,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J24)</f>
-        <v>0.183595551045647</v>
+        <v>0.187891959220834</v>
       </c>
       <c r="L24" s="15" t="n">
         <f aca="false">I24*K24</f>
-        <v>17267.7123624962</v>
+        <v>25373.6817410183</v>
       </c>
       <c r="M24" s="15" t="n">
         <f aca="false">B24*'Premissas Precept'!$B$15</f>
@@ -4748,23 +4748,23 @@
       </c>
       <c r="N24" s="15" t="n">
         <f aca="false">I24*'Premissas Precept'!$B$16</f>
-        <v>1881.06</v>
+        <v>2700.88</v>
       </c>
       <c r="O24" s="15" t="n">
         <f aca="false">(G24+H24)*'Premissas Precept'!$B$17</f>
-        <v>1949.55</v>
+        <v>3999.1</v>
       </c>
       <c r="P24" s="15" t="n">
         <f aca="false">(G24+H24)*'Premissas Precept'!$B$18</f>
-        <v>13646.85</v>
+        <v>27993.7</v>
       </c>
       <c r="Q24" s="15" t="n">
         <f aca="false">C24*'Premissas Precept'!$B$19+E24*'Premissas Precept'!$B$20</f>
-        <v>2400</v>
+        <v>4200</v>
       </c>
       <c r="R24" s="22" t="n">
         <f aca="false">SUM(L24:Q24)</f>
-        <v>41285.1723624962</v>
+        <v>68407.3617410183</v>
       </c>
       <c r="S24" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4772,19 +4772,19 @@
       </c>
       <c r="T24" s="15" t="n">
         <f aca="false">IF(A24&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I24,0)</f>
-        <v>19751.13</v>
+        <v>28359.24</v>
       </c>
       <c r="U24" s="22" t="n">
         <f aca="false">S24+T24</f>
-        <v>31751.13</v>
+        <v>40359.24</v>
       </c>
       <c r="V24" s="22" t="n">
         <f aca="false">I24-R24-U24</f>
-        <v>21016.6976375038</v>
+        <v>26277.3982589817</v>
       </c>
       <c r="W24" s="15" t="n">
         <f aca="false">T24/'Premissas Precept'!$B$45</f>
-        <v>2821.59</v>
+        <v>4051.32</v>
       </c>
       <c r="X24" s="35" t="str">
         <f aca="false">IF(V24&gt;=0,"Sim","Não")</f>
@@ -4799,7 +4799,7 @@
         <v>48</v>
       </c>
       <c r="C25" s="36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D25" s="36" t="n">
         <v>1</v>
@@ -4814,27 +4814,27 @@
       </c>
       <c r="G25" s="15" t="n">
         <f aca="false">C25*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>49985</v>
       </c>
       <c r="H25" s="15" t="n">
         <f aca="false">E25*'Premissas Precept'!$B$12</f>
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="I25" s="22" t="n">
         <f aca="false">F25+G25+H25</f>
-        <v>96447</v>
+        <v>137438</v>
       </c>
       <c r="J25" s="15" t="n">
         <f aca="false">SUM(I13:I24)</f>
-        <v>857046.166666667</v>
+        <v>1096834.5</v>
       </c>
       <c r="K25" s="38" t="n">
         <f aca="false">IF(J25&lt;=0,'Premissas Precept'!$C$24,(J25*LOOKUP(J25,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J25,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J25)</f>
-        <v>0.185047749275272</v>
+        <v>0.1894096807677</v>
       </c>
       <c r="L25" s="15" t="n">
         <f aca="false">I25*K25</f>
-        <v>17847.3002743522</v>
+        <v>26032.0877053512</v>
       </c>
       <c r="M25" s="15" t="n">
         <f aca="false">B25*'Premissas Precept'!$B$15</f>
@@ -4842,23 +4842,23 @@
       </c>
       <c r="N25" s="15" t="n">
         <f aca="false">I25*'Premissas Precept'!$B$16</f>
-        <v>1928.94</v>
+        <v>2748.76</v>
       </c>
       <c r="O25" s="15" t="n">
         <f aca="false">(G25+H25)*'Premissas Precept'!$B$17</f>
-        <v>1949.55</v>
+        <v>3999.1</v>
       </c>
       <c r="P25" s="15" t="n">
         <f aca="false">(G25+H25)*'Premissas Precept'!$B$18</f>
-        <v>13646.85</v>
+        <v>27993.7</v>
       </c>
       <c r="Q25" s="15" t="n">
         <f aca="false">C25*'Premissas Precept'!$B$19+E25*'Premissas Precept'!$B$20</f>
-        <v>2400</v>
+        <v>4200</v>
       </c>
       <c r="R25" s="22" t="n">
         <f aca="false">SUM(L25:Q25)</f>
-        <v>42092.6402743522</v>
+        <v>69293.6477053512</v>
       </c>
       <c r="S25" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4866,19 +4866,19 @@
       </c>
       <c r="T25" s="15" t="n">
         <f aca="false">IF(A25&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I25,0)</f>
-        <v>20253.87</v>
+        <v>28861.98</v>
       </c>
       <c r="U25" s="22" t="n">
         <f aca="false">S25+T25</f>
-        <v>32253.87</v>
+        <v>40861.98</v>
       </c>
       <c r="V25" s="22" t="n">
         <f aca="false">I25-R25-U25</f>
-        <v>22100.4897256478</v>
+        <v>27282.3722946488</v>
       </c>
       <c r="W25" s="15" t="n">
         <f aca="false">T25/'Premissas Precept'!$B$45</f>
-        <v>2893.41</v>
+        <v>4123.14</v>
       </c>
       <c r="X25" s="35" t="str">
         <f aca="false">IF(V25&gt;=0,"Sim","Não")</f>
@@ -4893,7 +4893,7 @@
         <v>50</v>
       </c>
       <c r="C26" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D26" s="36" t="n">
         <v>1</v>
@@ -4908,27 +4908,27 @@
       </c>
       <c r="G26" s="15" t="n">
         <f aca="false">C26*'Premissas Precept'!$B$9</f>
-        <v>29991</v>
+        <v>49985</v>
       </c>
       <c r="H26" s="15" t="n">
         <f aca="false">E26*'Premissas Precept'!$B$12</f>
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="I26" s="22" t="n">
         <f aca="false">F26+G26+H26</f>
-        <v>108838</v>
+        <v>139832</v>
       </c>
       <c r="J26" s="15" t="n">
         <f aca="false">SUM(I14:I25)</f>
-        <v>912026.833333333</v>
+        <v>1189139.5</v>
       </c>
       <c r="K26" s="38" t="n">
         <f aca="false">IF(J26&lt;=0,'Premissas Precept'!$C$24,(J26*LOOKUP(J26,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J26,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J26)</f>
-        <v>0.186250551655918</v>
+        <v>0.190619853684114</v>
       </c>
       <c r="L26" s="15" t="n">
         <f aca="false">I26*K26</f>
-        <v>20271.1375411268</v>
+        <v>26654.755380357</v>
       </c>
       <c r="M26" s="15" t="n">
         <f aca="false">B26*'Premissas Precept'!$B$15</f>
@@ -4936,23 +4936,23 @@
       </c>
       <c r="N26" s="15" t="n">
         <f aca="false">I26*'Premissas Precept'!$B$16</f>
-        <v>2176.76</v>
+        <v>2796.64</v>
       </c>
       <c r="O26" s="15" t="n">
         <f aca="false">(G26+H26)*'Premissas Precept'!$B$17</f>
-        <v>2449.4</v>
+        <v>3999.1</v>
       </c>
       <c r="P26" s="15" t="n">
         <f aca="false">(G26+H26)*'Premissas Precept'!$B$18</f>
-        <v>17145.8</v>
+        <v>27993.7</v>
       </c>
       <c r="Q26" s="15" t="n">
         <f aca="false">C26*'Premissas Precept'!$B$19+E26*'Premissas Precept'!$B$20</f>
-        <v>3000</v>
+        <v>4200</v>
       </c>
       <c r="R26" s="22" t="n">
         <f aca="false">SUM(L26:Q26)</f>
-        <v>49543.0975411268</v>
+        <v>70144.195380357</v>
       </c>
       <c r="S26" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -4960,19 +4960,19 @@
       </c>
       <c r="T26" s="15" t="n">
         <f aca="false">IF(A26&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I26,0)</f>
-        <v>22855.98</v>
+        <v>29364.72</v>
       </c>
       <c r="U26" s="22" t="n">
         <f aca="false">S26+T26</f>
-        <v>34855.98</v>
+        <v>41364.72</v>
       </c>
       <c r="V26" s="22" t="n">
         <f aca="false">I26-R26-U26</f>
-        <v>24438.9224588732</v>
+        <v>28323.084619643</v>
       </c>
       <c r="W26" s="15" t="n">
         <f aca="false">T26/'Premissas Precept'!$B$45</f>
-        <v>3265.14</v>
+        <v>4194.96</v>
       </c>
       <c r="X26" s="35" t="str">
         <f aca="false">IF(V26&gt;=0,"Sim","Não")</f>
@@ -4987,7 +4987,7 @@
         <v>52</v>
       </c>
       <c r="C27" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D27" s="36" t="n">
         <v>1</v>
@@ -5002,27 +5002,27 @@
       </c>
       <c r="G27" s="15" t="n">
         <f aca="false">C27*'Premissas Precept'!$B$9</f>
-        <v>29991</v>
+        <v>49985</v>
       </c>
       <c r="H27" s="15" t="n">
         <f aca="false">E27*'Premissas Precept'!$B$12</f>
-        <v>18997</v>
+        <v>29997</v>
       </c>
       <c r="I27" s="22" t="n">
         <f aca="false">F27+G27+H27</f>
-        <v>111232</v>
+        <v>142226</v>
       </c>
       <c r="J27" s="15" t="n">
         <f aca="false">SUM(I15:I26)</f>
-        <v>965810.5</v>
+        <v>1270250.5</v>
       </c>
       <c r="K27" s="38" t="n">
         <f aca="false">IF(J27&lt;=0,'Premissas Precept'!$C$24,(J27*LOOKUP(J27,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J27,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J27)</f>
-        <v>0.187294663394113</v>
+        <v>0.191538088353439</v>
       </c>
       <c r="L27" s="15" t="n">
         <f aca="false">I27*K27</f>
-        <v>20833.159998654</v>
+        <v>27241.6961541562</v>
       </c>
       <c r="M27" s="15" t="n">
         <f aca="false">B27*'Premissas Precept'!$B$15</f>
@@ -5030,23 +5030,23 @@
       </c>
       <c r="N27" s="15" t="n">
         <f aca="false">I27*'Premissas Precept'!$B$16</f>
-        <v>2224.64</v>
+        <v>2844.52</v>
       </c>
       <c r="O27" s="15" t="n">
         <f aca="false">(G27+H27)*'Premissas Precept'!$B$17</f>
-        <v>2449.4</v>
+        <v>3999.1</v>
       </c>
       <c r="P27" s="15" t="n">
         <f aca="false">(G27+H27)*'Premissas Precept'!$B$18</f>
-        <v>17145.8</v>
+        <v>27993.7</v>
       </c>
       <c r="Q27" s="15" t="n">
         <f aca="false">C27*'Premissas Precept'!$B$19+E27*'Premissas Precept'!$B$20</f>
-        <v>3000</v>
+        <v>4200</v>
       </c>
       <c r="R27" s="22" t="n">
         <f aca="false">SUM(L27:Q27)</f>
-        <v>50332.999998654</v>
+        <v>70959.0161541562</v>
       </c>
       <c r="S27" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -5054,19 +5054,19 @@
       </c>
       <c r="T27" s="15" t="n">
         <f aca="false">IF(A27&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I27,0)</f>
-        <v>23358.72</v>
+        <v>29867.46</v>
       </c>
       <c r="U27" s="22" t="n">
         <f aca="false">S27+T27</f>
-        <v>35358.72</v>
+        <v>41867.46</v>
       </c>
       <c r="V27" s="22" t="n">
         <f aca="false">I27-R27-U27</f>
-        <v>25540.280001346</v>
+        <v>29399.5238458438</v>
       </c>
       <c r="W27" s="15" t="n">
         <f aca="false">T27/'Premissas Precept'!$B$45</f>
-        <v>3336.96</v>
+        <v>4266.78</v>
       </c>
       <c r="X27" s="35" t="str">
         <f aca="false">IF(V27&gt;=0,"Sim","Não")</f>
@@ -5081,7 +5081,7 @@
         <v>54</v>
       </c>
       <c r="C28" s="36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D28" s="36" t="n">
         <v>0</v>
@@ -5096,27 +5096,27 @@
       </c>
       <c r="G28" s="15" t="n">
         <f aca="false">C28*'Premissas Precept'!$B$9</f>
-        <v>19994</v>
+        <v>49985</v>
       </c>
       <c r="H28" s="15" t="n">
         <f aca="false">E28*'Premissas Precept'!$B$12</f>
-        <v>15830.8333333333</v>
+        <v>24997.5</v>
       </c>
       <c r="I28" s="22" t="n">
         <f aca="false">F28+G28+H28</f>
-        <v>100462.833333333</v>
+        <v>139620.5</v>
       </c>
       <c r="J28" s="15" t="n">
         <f aca="false">SUM(I16:I27)</f>
-        <v>1026425</v>
+        <v>1356359</v>
       </c>
       <c r="K28" s="38" t="n">
         <f aca="false">IF(J28&lt;=0,'Premissas Precept'!$C$24,(J28*LOOKUP(J28,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J28,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J28)</f>
-        <v>0.188340234308401</v>
+        <v>0.192392718299506</v>
       </c>
       <c r="L28" s="15" t="n">
         <f aca="false">I28*K28</f>
-        <v>18921.1935692858</v>
+        <v>26861.9675253362</v>
       </c>
       <c r="M28" s="15" t="n">
         <f aca="false">B28*'Premissas Precept'!$B$15</f>
@@ -5124,23 +5124,23 @@
       </c>
       <c r="N28" s="15" t="n">
         <f aca="false">I28*'Premissas Precept'!$B$16</f>
-        <v>2009.25666666667</v>
+        <v>2792.41</v>
       </c>
       <c r="O28" s="15" t="n">
         <f aca="false">(G28+H28)*'Premissas Precept'!$B$17</f>
-        <v>1791.24166666667</v>
+        <v>3749.125</v>
       </c>
       <c r="P28" s="15" t="n">
         <f aca="false">(G28+H28)*'Premissas Precept'!$B$18</f>
-        <v>12538.6916666667</v>
+        <v>26243.875</v>
       </c>
       <c r="Q28" s="15" t="n">
         <f aca="false">C28*'Premissas Precept'!$B$19+E28*'Premissas Precept'!$B$20</f>
-        <v>2200</v>
+        <v>4000</v>
       </c>
       <c r="R28" s="22" t="n">
         <f aca="false">SUM(L28:Q28)</f>
-        <v>42320.3835692858</v>
+        <v>68507.3775253362</v>
       </c>
       <c r="S28" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -5148,19 +5148,19 @@
       </c>
       <c r="T28" s="15" t="n">
         <f aca="false">IF(A28&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I28,0)</f>
-        <v>21097.195</v>
+        <v>29320.305</v>
       </c>
       <c r="U28" s="22" t="n">
         <f aca="false">S28+T28</f>
-        <v>33097.195</v>
+        <v>41320.305</v>
       </c>
       <c r="V28" s="22" t="n">
         <f aca="false">I28-R28-U28</f>
-        <v>25045.2547640475</v>
+        <v>29792.8174746638</v>
       </c>
       <c r="W28" s="15" t="n">
         <f aca="false">T28/'Premissas Precept'!$B$45</f>
-        <v>3013.885</v>
+        <v>4188.615</v>
       </c>
       <c r="X28" s="35" t="str">
         <f aca="false">IF(V28&gt;=0,"Sim","Não")</f>
@@ -5175,7 +5175,7 @@
         <v>56</v>
       </c>
       <c r="C29" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D29" s="36" t="n">
         <v>1</v>
@@ -5190,27 +5190,27 @@
       </c>
       <c r="G29" s="15" t="n">
         <f aca="false">C29*'Premissas Precept'!$B$9</f>
-        <v>29991</v>
+        <v>49985</v>
       </c>
       <c r="H29" s="15" t="n">
         <f aca="false">E29*'Premissas Precept'!$B$12</f>
-        <v>15830.8333333333</v>
+        <v>24997.5</v>
       </c>
       <c r="I29" s="22" t="n">
         <f aca="false">F29+G29+H29</f>
-        <v>112853.833333333</v>
+        <v>142014.5</v>
       </c>
       <c r="J29" s="15" t="n">
         <f aca="false">SUM(I17:I28)</f>
-        <v>1062682.33333333</v>
+        <v>1426274</v>
       </c>
       <c r="K29" s="38" t="n">
         <f aca="false">IF(J29&lt;=0,'Premissas Precept'!$C$24,(J29*LOOKUP(J29,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$C$24:$C$29)-LOOKUP(J29,'Premissas Precept'!$B$24:$B$29,'Premissas Precept'!$D$24:$D$29))/J29)</f>
-        <v>0.188908643755879</v>
+        <v>0.193010718838035</v>
       </c>
       <c r="L29" s="15" t="n">
         <f aca="false">I29*K29</f>
-        <v>21319.0645976521</v>
+        <v>27410.3207304242</v>
       </c>
       <c r="M29" s="15" t="n">
         <f aca="false">B29*'Premissas Precept'!$B$15</f>
@@ -5218,23 +5218,23 @@
       </c>
       <c r="N29" s="15" t="n">
         <f aca="false">I29*'Premissas Precept'!$B$16</f>
-        <v>2257.07666666667</v>
+        <v>2840.29</v>
       </c>
       <c r="O29" s="15" t="n">
         <f aca="false">(G29+H29)*'Premissas Precept'!$B$17</f>
-        <v>2291.09166666667</v>
+        <v>3749.125</v>
       </c>
       <c r="P29" s="15" t="n">
         <f aca="false">(G29+H29)*'Premissas Precept'!$B$18</f>
-        <v>16037.6416666667</v>
+        <v>26243.875</v>
       </c>
       <c r="Q29" s="15" t="n">
         <f aca="false">C29*'Premissas Precept'!$B$19+E29*'Premissas Precept'!$B$20</f>
-        <v>2800</v>
+        <v>4000</v>
       </c>
       <c r="R29" s="22" t="n">
         <f aca="false">SUM(L29:Q29)</f>
-        <v>49744.8745976521</v>
+        <v>69283.6107304242</v>
       </c>
       <c r="S29" s="15" t="n">
         <f aca="false">'Premissas Precept'!$B$42</f>
@@ -5242,19 +5242,19 @@
       </c>
       <c r="T29" s="15" t="n">
         <f aca="false">IF(A29&gt;='Premissas Precept'!$B$47,'Premissas Precept'!$B$48*I29,0)</f>
-        <v>23699.305</v>
+        <v>29823.045</v>
       </c>
       <c r="U29" s="22" t="n">
         <f aca="false">S29+T29</f>
-        <v>35699.305</v>
+        <v>41823.045</v>
       </c>
       <c r="V29" s="22" t="n">
         <f aca="false">I29-R29-U29</f>
-        <v>27409.6537356813</v>
+        <v>30907.8442695758</v>
       </c>
       <c r="W29" s="15" t="n">
         <f aca="false">T29/'Premissas Precept'!$B$45</f>
-        <v>3385.615</v>
+        <v>4260.435</v>
       </c>
       <c r="X29" s="35" t="str">
         <f aca="false">IF(V29&gt;=0,"Sim","Não")</f>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="C30" s="40" t="n">
         <f aca="false">SUM(C6:C29)</f>
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="D30" s="40" t="n">
         <f aca="false">SUM(D6:D29)</f>
@@ -5284,21 +5284,21 @@
       </c>
       <c r="G30" s="22" t="n">
         <f aca="false">SUM(G6:G29)</f>
-        <v>379886</v>
+        <v>649805</v>
       </c>
       <c r="H30" s="22" t="n">
         <f aca="false">SUM(H6:H29)</f>
-        <v>250127.166666667</v>
+        <v>394960.5</v>
       </c>
       <c r="I30" s="22" t="n">
         <f aca="false">SUM(I6:I29)</f>
-        <v>1527763.16666667</v>
+        <v>1942515.5</v>
       </c>
       <c r="J30" s="32"/>
       <c r="K30" s="32"/>
       <c r="L30" s="22" t="n">
         <f aca="false">SUM(L6:L29)</f>
-        <v>270672.002691224</v>
+        <v>351518.004455835</v>
       </c>
       <c r="M30" s="22" t="n">
         <f aca="false">SUM(M6:M29)</f>
@@ -5306,23 +5306,23 @@
       </c>
       <c r="N30" s="22" t="n">
         <f aca="false">SUM(N6:N29)</f>
-        <v>30555.2633333333</v>
+        <v>38850.31</v>
       </c>
       <c r="O30" s="22" t="n">
         <f aca="false">SUM(O6:O29)</f>
-        <v>31500.6583333333</v>
+        <v>52238.275</v>
       </c>
       <c r="P30" s="22" t="n">
         <f aca="false">SUM(P6:P29)</f>
-        <v>220504.608333333</v>
+        <v>365667.925</v>
       </c>
       <c r="Q30" s="22" t="n">
         <f aca="false">SUM(Q6:Q29)</f>
-        <v>38600</v>
+        <v>54800</v>
       </c>
       <c r="R30" s="22" t="n">
         <f aca="false">SUM(R6:R29)</f>
-        <v>659332.532691224</v>
+        <v>930574.514455835</v>
       </c>
       <c r="S30" s="22" t="n">
         <f aca="false">SUM(S6:S29)</f>
@@ -5330,19 +5330,19 @@
       </c>
       <c r="T30" s="22" t="n">
         <f aca="false">SUM(T6:T29)</f>
-        <v>316054.235</v>
+        <v>403152.225</v>
       </c>
       <c r="U30" s="22" t="n">
         <f aca="false">SUM(U6:U29)</f>
-        <v>604054.235</v>
+        <v>691152.225</v>
       </c>
       <c r="V30" s="22" t="n">
         <f aca="false">SUM(V6:V29)</f>
-        <v>264376.398975443</v>
+        <v>320788.760544165</v>
       </c>
       <c r="W30" s="22" t="n">
         <f aca="false">SUM(W6:W29)</f>
-        <v>45150.605</v>
+        <v>57593.175</v>
       </c>
       <c r="X30" s="32"/>
     </row>
@@ -5427,26 +5427,26 @@
       <c r="D35" s="43"/>
       <c r="E35" s="28" t="n">
         <f aca="false">AVERAGE(I6:I11)</f>
-        <v>17496.1944444444</v>
+        <v>17801.75</v>
       </c>
       <c r="F35" s="28" t="n">
         <f aca="false">AVERAGE(R6:R11)</f>
-        <v>6505.64513888889</v>
+        <v>6681.33958333333</v>
       </c>
       <c r="G35" s="28" t="n">
         <f aca="false">AVERAGE(U6:U11)</f>
-        <v>14878.1958333333</v>
+        <v>14942.3625</v>
       </c>
       <c r="H35" s="15" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="23" t="n">
         <f aca="false">F35/E35</f>
-        <v>0.371832009500479</v>
+        <v>0.375319257001887</v>
       </c>
       <c r="J35" s="15" t="n">
         <f aca="false">E35-F35-G35</f>
-        <v>-3887.64652777778</v>
+        <v>-3821.95208333333</v>
       </c>
       <c r="K35" s="44" t="n">
         <f aca="false">AVERAGE(B6:B11)</f>
@@ -5472,26 +5472,26 @@
       <c r="D36" s="43"/>
       <c r="E36" s="28" t="n">
         <f aca="false">AVERAGE(I12:I17)</f>
-        <v>50642.0555555556</v>
+        <v>54919.8333333333</v>
       </c>
       <c r="F36" s="28" t="n">
         <f aca="false">AVERAGE(R12:R17)</f>
-        <v>21163.1004869335</v>
+        <v>23711.3861311891</v>
       </c>
       <c r="G36" s="28" t="n">
         <f aca="false">AVERAGE(U12:U17)</f>
-        <v>22634.8316666667</v>
+        <v>23533.165</v>
       </c>
       <c r="H36" s="15" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="23" t="n">
         <f aca="false">F36/E36</f>
-        <v>0.417895763802815</v>
+        <v>0.431745413123779</v>
       </c>
       <c r="J36" s="15" t="n">
         <f aca="false">E36-F36-G36</f>
-        <v>6844.12340195541</v>
+        <v>7675.28220214424</v>
       </c>
       <c r="K36" s="44" t="n">
         <f aca="false">AVERAGE(B12:B17)</f>
@@ -5517,26 +5517,26 @@
       <c r="D37" s="43"/>
       <c r="E37" s="28" t="n">
         <f aca="false">AVERAGE(I18:I29)</f>
-        <v>93244.4722222222</v>
+        <v>125515.5</v>
       </c>
       <c r="F37" s="28" t="n">
         <f aca="false">AVERAGE(R18:R29)</f>
-        <v>41110.0049113575</v>
+        <v>62351.5133473917</v>
       </c>
       <c r="G37" s="28" t="n">
         <f aca="false">AVERAGE(U18:U29)</f>
-        <v>31581.3391666667</v>
+        <v>38358.255</v>
       </c>
       <c r="H37" s="15" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="23" t="n">
         <f aca="false">F37/E37</f>
-        <v>0.440884096736407</v>
+        <v>0.496763454293627</v>
       </c>
       <c r="J37" s="15" t="n">
         <f aca="false">E37-F37-G37</f>
-        <v>20553.1281441981</v>
+        <v>24805.7316526083</v>
       </c>
       <c r="K37" s="44" t="n">
         <f aca="false">AVERAGE(B18:B29)</f>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="L37" s="34" t="n">
         <f aca="false">SUM(C18:C29)</f>
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="M37" s="34" t="n">
         <f aca="false">SUM(D18:D29)</f>
@@ -5622,7 +5622,7 @@
       <c r="D44" s="45"/>
       <c r="E44" s="44" t="n">
         <f aca="false">AVERAGE(C18:C29)</f>
-        <v>2.25</v>
+        <v>4.5</v>
       </c>
       <c r="F44" s="15" t="n">
         <f aca="false">'Premissas Precept'!B9</f>
@@ -5630,7 +5630,7 @@
       </c>
       <c r="G44" s="15" t="n">
         <f aca="false">E44*F44</f>
-        <v>22493.25</v>
+        <v>44986.5</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5646,11 +5646,11 @@
       </c>
       <c r="F45" s="15" t="n">
         <f aca="false">'Premissas Precept'!B12</f>
-        <v>3166.16666666667</v>
+        <v>4999.5</v>
       </c>
       <c r="G45" s="15" t="n">
         <f aca="false">E45*F45</f>
-        <v>16886.2222222222</v>
+        <v>26664</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5664,7 +5664,7 @@
       <c r="F46" s="15"/>
       <c r="G46" s="28" t="n">
         <f aca="false">SUM(G42:G45)</f>
-        <v>93244.4722222222</v>
+        <v>125515.5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5697,11 +5697,11 @@
       <c r="E48" s="44"/>
       <c r="F48" s="23" t="n">
         <f aca="false">G48/G46</f>
-        <v>0.182602351705945</v>
+        <v>0.186147023122443</v>
       </c>
       <c r="G48" s="15" t="n">
         <f aca="false">AVERAGE(L18:L29)</f>
-        <v>17026.6599113575</v>
+        <v>23364.3366807251</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="G49" s="15" t="n">
         <f aca="false">AVERAGE(N18:N29)</f>
-        <v>1864.88944444444</v>
+        <v>2510.31</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="G50" s="15" t="n">
         <f aca="false">AVERAGE(O18:O29)</f>
-        <v>1968.97361111111</v>
+        <v>3582.525</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5749,7 +5749,7 @@
       <c r="F51" s="15"/>
       <c r="G51" s="15" t="n">
         <f aca="false">AVERAGE(Q18:Q29)</f>
-        <v>2416.66666666667</v>
+        <v>3766.66666666667</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="G52" s="15" t="n">
         <f aca="false">AVERAGE(P18:P29)</f>
-        <v>13782.8152777778</v>
+        <v>25077.675</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5779,11 +5779,11 @@
       <c r="E53" s="44"/>
       <c r="F53" s="23" t="n">
         <f aca="false">G53/G46</f>
-        <v>0.440884096736408</v>
+        <v>0.496763454293627</v>
       </c>
       <c r="G53" s="28" t="n">
         <f aca="false">SUM(G47:G52)</f>
-        <v>41110.0049113575</v>
+        <v>62351.5133473917</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="G54" s="15" t="n">
         <f aca="false">AVERAGE(T18:T29)</f>
-        <v>19581.3391666667</v>
+        <v>26358.255</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5828,7 +5828,7 @@
       <c r="F56" s="15"/>
       <c r="G56" s="28" t="n">
         <f aca="false">G54+G55</f>
-        <v>31581.3391666667</v>
+        <v>38358.255</v>
       </c>
     </row>
   </sheetData>
@@ -6083,24 +6083,24 @@
       </c>
       <c r="B11" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I11</f>
-        <v>32315.1666666667</v>
+        <v>34148.5</v>
       </c>
       <c r="C11" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R11</f>
-        <v>13160.4208333333</v>
+        <v>14214.5875</v>
       </c>
       <c r="D11" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U11</f>
-        <v>18786.185</v>
+        <v>19171.185</v>
       </c>
       <c r="E11" s="51" t="n">
         <f aca="false">B11-C11-D11</f>
-        <v>368.560833333333</v>
+        <v>762.727500000001</v>
       </c>
       <c r="F11" s="50"/>
       <c r="G11" s="52" t="n">
         <f aca="false">E11-F11</f>
-        <v>368.560833333333</v>
+        <v>762.727500000001</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6109,24 +6109,24 @@
       </c>
       <c r="B12" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I12</f>
-        <v>35906.1666666667</v>
+        <v>37739.5</v>
       </c>
       <c r="C12" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R12</f>
-        <v>14186.9147886128</v>
+        <v>15261.5044237224</v>
       </c>
       <c r="D12" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U12</f>
-        <v>19540.295</v>
+        <v>19925.295</v>
       </c>
       <c r="E12" s="51" t="n">
         <f aca="false">B12-C12-D12</f>
-        <v>2178.95687805391</v>
+        <v>2552.70057627762</v>
       </c>
       <c r="F12" s="50"/>
       <c r="G12" s="52" t="n">
         <f aca="false">E12-F12</f>
-        <v>2178.95687805391</v>
+        <v>2552.70057627762</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6135,24 +6135,24 @@
       </c>
       <c r="B13" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I13</f>
-        <v>41466.3333333333</v>
+        <v>45133</v>
       </c>
       <c r="C13" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R13</f>
-        <v>16942.3811072992</v>
+        <v>19095.3934624697</v>
       </c>
       <c r="D13" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U13</f>
-        <v>20707.93</v>
+        <v>21477.93</v>
       </c>
       <c r="E13" s="51" t="n">
         <f aca="false">B13-C13-D13</f>
-        <v>3816.02222603415</v>
+        <v>4559.67653753027</v>
       </c>
       <c r="F13" s="50"/>
       <c r="G13" s="52" t="n">
         <f aca="false">E13-F13</f>
-        <v>3816.02222603415</v>
+        <v>4559.67653753027</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6161,24 +6161,24 @@
       </c>
       <c r="B14" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I14</f>
-        <v>55054.3333333333</v>
+        <v>58721</v>
       </c>
       <c r="C14" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R14</f>
-        <v>24395.6511548326</v>
+        <v>26572.6768144747</v>
       </c>
       <c r="D14" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U14</f>
-        <v>23561.41</v>
+        <v>24331.41</v>
       </c>
       <c r="E14" s="51" t="n">
         <f aca="false">B14-C14-D14</f>
-        <v>7097.27217850077</v>
+        <v>7816.91318552533</v>
       </c>
       <c r="F14" s="50"/>
       <c r="G14" s="52" t="n">
         <f aca="false">E14-F14</f>
-        <v>7097.27217850077</v>
+        <v>7816.91318552533</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6187,24 +6187,24 @@
       </c>
       <c r="B15" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I15</f>
-        <v>50617.5</v>
+        <v>56117.5</v>
       </c>
       <c r="C15" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R15</f>
-        <v>20742.1078174757</v>
+        <v>23999.2462452295</v>
       </c>
       <c r="D15" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U15</f>
-        <v>22629.675</v>
+        <v>23784.675</v>
       </c>
       <c r="E15" s="51" t="n">
         <f aca="false">B15-C15-D15</f>
-        <v>7245.71718252431</v>
+        <v>8333.57875477045</v>
       </c>
       <c r="F15" s="50"/>
       <c r="G15" s="52" t="n">
         <f aca="false">E15-F15</f>
-        <v>7245.71718252431</v>
+        <v>8333.57875477045</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6213,24 +6213,24 @@
       </c>
       <c r="B16" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I16</f>
-        <v>64205.5</v>
+        <v>69705.5</v>
       </c>
       <c r="C16" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R16</f>
-        <v>28212.1532911606</v>
+        <v>31505.2431779817</v>
       </c>
       <c r="D16" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U16</f>
-        <v>25483.155</v>
+        <v>26638.155</v>
       </c>
       <c r="E16" s="51" t="n">
         <f aca="false">B16-C16-D16</f>
-        <v>10510.1917088394</v>
+        <v>11562.1018220183</v>
       </c>
       <c r="F16" s="50"/>
       <c r="G16" s="52" t="n">
         <f aca="false">E16-F16</f>
-        <v>10510.1917088394</v>
+        <v>11562.1018220183</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6239,24 +6239,24 @@
       </c>
       <c r="B17" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I17</f>
-        <v>56602.5</v>
+        <v>62102.5</v>
       </c>
       <c r="C17" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R17</f>
-        <v>22499.3947622201</v>
+        <v>25834.2526632565</v>
       </c>
       <c r="D17" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U17</f>
-        <v>23886.525</v>
+        <v>25041.525</v>
       </c>
       <c r="E17" s="51" t="n">
         <f aca="false">B17-C17-D17</f>
-        <v>10216.5802377799</v>
+        <v>11226.7223367435</v>
       </c>
       <c r="F17" s="50"/>
       <c r="G17" s="52" t="n">
         <f aca="false">E17-F17</f>
-        <v>10216.5802377799</v>
+        <v>11226.7223367435</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6265,24 +6265,24 @@
       </c>
       <c r="B18" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I18</f>
-        <v>73356.6666666667</v>
+        <v>100684</v>
       </c>
       <c r="C18" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R18</f>
-        <v>32118.783568517</v>
+        <v>49617.013039618</v>
       </c>
       <c r="D18" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U18</f>
-        <v>27404.9</v>
+        <v>33143.64</v>
       </c>
       <c r="E18" s="51" t="n">
         <f aca="false">B18-C18-D18</f>
-        <v>13832.9830981497</v>
+        <v>17923.346960382</v>
       </c>
       <c r="F18" s="50"/>
       <c r="G18" s="52" t="n">
         <f aca="false">E18-F18</f>
-        <v>13832.9830981497</v>
+        <v>17923.346960382</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6291,24 +6291,24 @@
       </c>
       <c r="B19" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I19</f>
-        <v>75750.6666666667</v>
+        <v>103078</v>
       </c>
       <c r="C19" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R19</f>
-        <v>33018.9876080169</v>
+        <v>50678.801891933</v>
       </c>
       <c r="D19" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U19</f>
-        <v>27907.64</v>
+        <v>33646.38</v>
       </c>
       <c r="E19" s="51" t="n">
         <f aca="false">B19-C19-D19</f>
-        <v>14824.0390586497</v>
+        <v>18752.818108067</v>
       </c>
       <c r="F19" s="50"/>
       <c r="G19" s="52" t="n">
         <f aca="false">E19-F19</f>
-        <v>14824.0390586497</v>
+        <v>18752.818108067</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6317,24 +6317,24 @@
       </c>
       <c r="B20" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I20</f>
-        <v>81310.8333333333</v>
+        <v>110471.5</v>
       </c>
       <c r="C20" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R20</f>
-        <v>35957.3556297414</v>
+        <v>54824.4000516759</v>
       </c>
       <c r="D20" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U20</f>
-        <v>29075.275</v>
+        <v>35199.015</v>
       </c>
       <c r="E20" s="51" t="n">
         <f aca="false">B20-C20-D20</f>
-        <v>16278.2027035919</v>
+        <v>20448.0849483241</v>
       </c>
       <c r="F20" s="50"/>
       <c r="G20" s="52" t="n">
         <f aca="false">E20-F20</f>
-        <v>16278.2027035919</v>
+        <v>20448.0849483241</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6343,24 +6343,24 @@
       </c>
       <c r="B21" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I21</f>
-        <v>83704.8333333333</v>
+        <v>112865.5</v>
       </c>
       <c r="C21" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R21</f>
-        <v>36782.3174679213</v>
+        <v>55737.1828766041</v>
       </c>
       <c r="D21" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U21</f>
-        <v>29578.015</v>
+        <v>35701.755</v>
       </c>
       <c r="E21" s="51" t="n">
         <f aca="false">B21-C21-D21</f>
-        <v>17344.500865412</v>
+        <v>21426.5621233959</v>
       </c>
       <c r="F21" s="50"/>
       <c r="G21" s="52" t="n">
         <f aca="false">E21-F21</f>
-        <v>17344.500865412</v>
+        <v>21426.5621233959</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6369,24 +6369,24 @@
       </c>
       <c r="B22" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I22</f>
-        <v>89265</v>
+        <v>120259</v>
       </c>
       <c r="C22" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R22</f>
-        <v>39663.1104350631</v>
+        <v>59916.8317975888</v>
       </c>
       <c r="D22" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U22</f>
-        <v>30745.65</v>
+        <v>37254.39</v>
       </c>
       <c r="E22" s="51" t="n">
         <f aca="false">B22-C22-D22</f>
-        <v>18856.2395649369</v>
+        <v>23087.7782024112</v>
       </c>
       <c r="F22" s="50"/>
       <c r="G22" s="52" t="n">
         <f aca="false">E22-F22</f>
-        <v>18856.2395649369</v>
+        <v>23087.7782024112</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6395,24 +6395,24 @@
       </c>
       <c r="B23" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I23</f>
-        <v>91659</v>
+        <v>122653</v>
       </c>
       <c r="C23" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R23</f>
-        <v>40460.3358834631</v>
+        <v>60848.7212746378</v>
       </c>
       <c r="D23" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U23</f>
-        <v>31248.39</v>
+        <v>37757.13</v>
       </c>
       <c r="E23" s="51" t="n">
         <f aca="false">B23-C23-D23</f>
-        <v>19950.2741165369</v>
+        <v>24047.1487253622</v>
       </c>
       <c r="F23" s="50"/>
       <c r="G23" s="52" t="n">
         <f aca="false">E23-F23</f>
-        <v>19950.2741165369</v>
+        <v>24047.1487253622</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6421,24 +6421,24 @@
       </c>
       <c r="B24" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I24</f>
-        <v>94053</v>
+        <v>135044</v>
       </c>
       <c r="C24" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R24</f>
-        <v>41285.1723624962</v>
+        <v>68407.3617410183</v>
       </c>
       <c r="D24" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U24</f>
-        <v>31751.13</v>
+        <v>40359.24</v>
       </c>
       <c r="E24" s="51" t="n">
         <f aca="false">B24-C24-D24</f>
-        <v>21016.6976375038</v>
+        <v>26277.3982589817</v>
       </c>
       <c r="F24" s="50"/>
       <c r="G24" s="52" t="n">
         <f aca="false">E24-F24</f>
-        <v>21016.6976375038</v>
+        <v>26277.3982589817</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6447,24 +6447,24 @@
       </c>
       <c r="B25" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I25</f>
-        <v>96447</v>
+        <v>137438</v>
       </c>
       <c r="C25" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R25</f>
-        <v>42092.6402743522</v>
+        <v>69293.6477053512</v>
       </c>
       <c r="D25" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U25</f>
-        <v>32253.87</v>
+        <v>40861.98</v>
       </c>
       <c r="E25" s="51" t="n">
         <f aca="false">B25-C25-D25</f>
-        <v>22100.4897256478</v>
+        <v>27282.3722946488</v>
       </c>
       <c r="F25" s="50"/>
       <c r="G25" s="52" t="n">
         <f aca="false">E25-F25</f>
-        <v>22100.4897256478</v>
+        <v>27282.3722946488</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6473,24 +6473,24 @@
       </c>
       <c r="B26" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I26</f>
-        <v>108838</v>
+        <v>139832</v>
       </c>
       <c r="C26" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R26</f>
-        <v>49543.0975411268</v>
+        <v>70144.195380357</v>
       </c>
       <c r="D26" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U26</f>
-        <v>34855.98</v>
+        <v>41364.72</v>
       </c>
       <c r="E26" s="51" t="n">
         <f aca="false">B26-C26-D26</f>
-        <v>24438.9224588732</v>
+        <v>28323.084619643</v>
       </c>
       <c r="F26" s="50"/>
       <c r="G26" s="52" t="n">
         <f aca="false">E26-F26</f>
-        <v>24438.9224588732</v>
+        <v>28323.084619643</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6499,24 +6499,24 @@
       </c>
       <c r="B27" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I27</f>
-        <v>111232</v>
+        <v>142226</v>
       </c>
       <c r="C27" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R27</f>
-        <v>50332.999998654</v>
+        <v>70959.0161541562</v>
       </c>
       <c r="D27" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U27</f>
-        <v>35358.72</v>
+        <v>41867.46</v>
       </c>
       <c r="E27" s="51" t="n">
         <f aca="false">B27-C27-D27</f>
-        <v>25540.280001346</v>
+        <v>29399.5238458438</v>
       </c>
       <c r="F27" s="50"/>
       <c r="G27" s="52" t="n">
         <f aca="false">E27-F27</f>
-        <v>25540.280001346</v>
+        <v>29399.5238458438</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6525,24 +6525,24 @@
       </c>
       <c r="B28" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I28</f>
-        <v>100462.833333333</v>
+        <v>139620.5</v>
       </c>
       <c r="C28" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R28</f>
-        <v>42320.3835692858</v>
+        <v>68507.3775253362</v>
       </c>
       <c r="D28" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U28</f>
-        <v>33097.195</v>
+        <v>41320.305</v>
       </c>
       <c r="E28" s="51" t="n">
         <f aca="false">B28-C28-D28</f>
-        <v>25045.2547640475</v>
+        <v>29792.8174746638</v>
       </c>
       <c r="F28" s="50"/>
       <c r="G28" s="52" t="n">
         <f aca="false">E28-F28</f>
-        <v>25045.2547640475</v>
+        <v>29792.8174746638</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6551,24 +6551,24 @@
       </c>
       <c r="B29" s="50" t="n">
         <f aca="false">'Projeção Mensal'!I29</f>
-        <v>112853.833333333</v>
+        <v>142014.5</v>
       </c>
       <c r="C29" s="50" t="n">
         <f aca="false">'Projeção Mensal'!R29</f>
-        <v>49744.8745976521</v>
+        <v>69283.6107304242</v>
       </c>
       <c r="D29" s="50" t="n">
         <f aca="false">'Projeção Mensal'!U29</f>
-        <v>35699.305</v>
+        <v>41823.045</v>
       </c>
       <c r="E29" s="51" t="n">
         <f aca="false">B29-C29-D29</f>
-        <v>27409.6537356813</v>
+        <v>30907.8442695758</v>
       </c>
       <c r="F29" s="50"/>
       <c r="G29" s="52" t="n">
         <f aca="false">E29-F29</f>
-        <v>27409.6537356813</v>
+        <v>30907.8442695758</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6577,19 +6577,19 @@
       </c>
       <c r="B30" s="52" t="n">
         <f aca="false">SUM(B5:B29)</f>
-        <v>1527763.16666667</v>
+        <v>1942515.5</v>
       </c>
       <c r="C30" s="52" t="n">
         <f aca="false">SUM(C5:C29)</f>
-        <v>659332.532691224</v>
+        <v>930574.514455835</v>
       </c>
       <c r="D30" s="52" t="n">
         <f aca="false">SUM(D5:D29)</f>
-        <v>604054.235</v>
+        <v>691152.225</v>
       </c>
       <c r="E30" s="52" t="n">
         <f aca="false">SUM(E5:E29)</f>
-        <v>264376.398975443</v>
+        <v>320788.760544165</v>
       </c>
       <c r="F30" s="52" t="n">
         <f aca="false">SUM(F5:F29)</f>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="G30" s="52" t="n">
         <f aca="false">SUM(G5:G29)</f>
-        <v>162376.398975443</v>
+        <v>218788.760544165</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6879,15 +6879,15 @@
       </c>
       <c r="B11" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B11</f>
-        <v>32315.1666666667</v>
+        <v>34148.5</v>
       </c>
       <c r="C11" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C11</f>
-        <v>13160.4208333333</v>
+        <v>14214.5875</v>
       </c>
       <c r="D11" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D11</f>
-        <v>18786.185</v>
+        <v>19171.185</v>
       </c>
       <c r="E11" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F11</f>
@@ -6895,11 +6895,11 @@
       </c>
       <c r="F11" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>368.560833333333</v>
+        <v>762.727500000001</v>
       </c>
       <c r="G11" s="52" t="n">
         <f aca="false">G10+F11</f>
-        <v>-125325.879166667</v>
+        <v>-124931.7125</v>
       </c>
       <c r="H11" s="55" t="str">
         <f aca="false">IF(G11&gt;=0,"Sim","Não")</f>
@@ -6912,15 +6912,15 @@
       </c>
       <c r="B12" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B12</f>
-        <v>35906.1666666667</v>
+        <v>37739.5</v>
       </c>
       <c r="C12" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C12</f>
-        <v>14186.9147886128</v>
+        <v>15261.5044237224</v>
       </c>
       <c r="D12" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D12</f>
-        <v>19540.295</v>
+        <v>19925.295</v>
       </c>
       <c r="E12" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F12</f>
@@ -6928,11 +6928,11 @@
       </c>
       <c r="F12" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>2178.95687805391</v>
+        <v>2552.70057627762</v>
       </c>
       <c r="G12" s="52" t="n">
         <f aca="false">G11+F12</f>
-        <v>-123146.922288613</v>
+        <v>-122379.011923722</v>
       </c>
       <c r="H12" s="55" t="str">
         <f aca="false">IF(G12&gt;=0,"Sim","Não")</f>
@@ -6945,15 +6945,15 @@
       </c>
       <c r="B13" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B13</f>
-        <v>41466.3333333333</v>
+        <v>45133</v>
       </c>
       <c r="C13" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C13</f>
-        <v>16942.3811072992</v>
+        <v>19095.3934624697</v>
       </c>
       <c r="D13" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D13</f>
-        <v>20707.93</v>
+        <v>21477.93</v>
       </c>
       <c r="E13" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F13</f>
@@ -6961,11 +6961,11 @@
       </c>
       <c r="F13" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>3816.02222603415</v>
+        <v>4559.67653753027</v>
       </c>
       <c r="G13" s="52" t="n">
         <f aca="false">G12+F13</f>
-        <v>-119330.900062579</v>
+        <v>-117819.335386192</v>
       </c>
       <c r="H13" s="55" t="str">
         <f aca="false">IF(G13&gt;=0,"Sim","Não")</f>
@@ -6978,15 +6978,15 @@
       </c>
       <c r="B14" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B14</f>
-        <v>55054.3333333333</v>
+        <v>58721</v>
       </c>
       <c r="C14" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C14</f>
-        <v>24395.6511548326</v>
+        <v>26572.6768144747</v>
       </c>
       <c r="D14" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D14</f>
-        <v>23561.41</v>
+        <v>24331.41</v>
       </c>
       <c r="E14" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F14</f>
@@ -6994,11 +6994,11 @@
       </c>
       <c r="F14" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>7097.27217850077</v>
+        <v>7816.91318552533</v>
       </c>
       <c r="G14" s="52" t="n">
         <f aca="false">G13+F14</f>
-        <v>-112233.627884078</v>
+        <v>-110002.422200667</v>
       </c>
       <c r="H14" s="55" t="str">
         <f aca="false">IF(G14&gt;=0,"Sim","Não")</f>
@@ -7011,15 +7011,15 @@
       </c>
       <c r="B15" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B15</f>
-        <v>50617.5</v>
+        <v>56117.5</v>
       </c>
       <c r="C15" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C15</f>
-        <v>20742.1078174757</v>
+        <v>23999.2462452295</v>
       </c>
       <c r="D15" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D15</f>
-        <v>22629.675</v>
+        <v>23784.675</v>
       </c>
       <c r="E15" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F15</f>
@@ -7027,11 +7027,11 @@
       </c>
       <c r="F15" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>7245.71718252431</v>
+        <v>8333.57875477045</v>
       </c>
       <c r="G15" s="52" t="n">
         <f aca="false">G14+F15</f>
-        <v>-104987.910701554</v>
+        <v>-101668.843445896</v>
       </c>
       <c r="H15" s="55" t="str">
         <f aca="false">IF(G15&gt;=0,"Sim","Não")</f>
@@ -7044,15 +7044,15 @@
       </c>
       <c r="B16" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B16</f>
-        <v>64205.5</v>
+        <v>69705.5</v>
       </c>
       <c r="C16" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C16</f>
-        <v>28212.1532911606</v>
+        <v>31505.2431779817</v>
       </c>
       <c r="D16" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D16</f>
-        <v>25483.155</v>
+        <v>26638.155</v>
       </c>
       <c r="E16" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F16</f>
@@ -7060,11 +7060,11 @@
       </c>
       <c r="F16" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>10510.1917088394</v>
+        <v>11562.1018220183</v>
       </c>
       <c r="G16" s="52" t="n">
         <f aca="false">G15+F16</f>
-        <v>-94477.7189927141</v>
+        <v>-90106.741623878</v>
       </c>
       <c r="H16" s="55" t="str">
         <f aca="false">IF(G16&gt;=0,"Sim","Não")</f>
@@ -7077,15 +7077,15 @@
       </c>
       <c r="B17" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B17</f>
-        <v>56602.5</v>
+        <v>62102.5</v>
       </c>
       <c r="C17" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C17</f>
-        <v>22499.3947622201</v>
+        <v>25834.2526632565</v>
       </c>
       <c r="D17" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D17</f>
-        <v>23886.525</v>
+        <v>25041.525</v>
       </c>
       <c r="E17" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F17</f>
@@ -7093,11 +7093,11 @@
       </c>
       <c r="F17" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>10216.5802377799</v>
+        <v>11226.7223367435</v>
       </c>
       <c r="G17" s="52" t="n">
         <f aca="false">G16+F17</f>
-        <v>-84261.1387549342</v>
+        <v>-78880.0192871346</v>
       </c>
       <c r="H17" s="55" t="str">
         <f aca="false">IF(G17&gt;=0,"Sim","Não")</f>
@@ -7110,15 +7110,15 @@
       </c>
       <c r="B18" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B18</f>
-        <v>73356.6666666667</v>
+        <v>100684</v>
       </c>
       <c r="C18" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C18</f>
-        <v>32118.783568517</v>
+        <v>49617.013039618</v>
       </c>
       <c r="D18" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D18</f>
-        <v>27404.9</v>
+        <v>33143.64</v>
       </c>
       <c r="E18" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F18</f>
@@ -7126,11 +7126,11 @@
       </c>
       <c r="F18" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>13832.9830981497</v>
+        <v>17923.346960382</v>
       </c>
       <c r="G18" s="52" t="n">
         <f aca="false">G17+F18</f>
-        <v>-70428.1556567845</v>
+        <v>-60956.6723267525</v>
       </c>
       <c r="H18" s="55" t="str">
         <f aca="false">IF(G18&gt;=0,"Sim","Não")</f>
@@ -7143,15 +7143,15 @@
       </c>
       <c r="B19" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B19</f>
-        <v>75750.6666666667</v>
+        <v>103078</v>
       </c>
       <c r="C19" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C19</f>
-        <v>33018.9876080169</v>
+        <v>50678.801891933</v>
       </c>
       <c r="D19" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D19</f>
-        <v>27907.64</v>
+        <v>33646.38</v>
       </c>
       <c r="E19" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F19</f>
@@ -7159,11 +7159,11 @@
       </c>
       <c r="F19" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>14824.0390586497</v>
+        <v>18752.818108067</v>
       </c>
       <c r="G19" s="52" t="n">
         <f aca="false">G18+F19</f>
-        <v>-55604.1165981347</v>
+        <v>-42203.8542186856</v>
       </c>
       <c r="H19" s="55" t="str">
         <f aca="false">IF(G19&gt;=0,"Sim","Não")</f>
@@ -7176,15 +7176,15 @@
       </c>
       <c r="B20" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B20</f>
-        <v>81310.8333333333</v>
+        <v>110471.5</v>
       </c>
       <c r="C20" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C20</f>
-        <v>35957.3556297414</v>
+        <v>54824.4000516759</v>
       </c>
       <c r="D20" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D20</f>
-        <v>29075.275</v>
+        <v>35199.015</v>
       </c>
       <c r="E20" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F20</f>
@@ -7192,11 +7192,11 @@
       </c>
       <c r="F20" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>16278.2027035919</v>
+        <v>20448.0849483241</v>
       </c>
       <c r="G20" s="52" t="n">
         <f aca="false">G19+F20</f>
-        <v>-39325.9138945428</v>
+        <v>-21755.7692703615</v>
       </c>
       <c r="H20" s="55" t="str">
         <f aca="false">IF(G20&gt;=0,"Sim","Não")</f>
@@ -7209,15 +7209,15 @@
       </c>
       <c r="B21" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B21</f>
-        <v>83704.8333333333</v>
+        <v>112865.5</v>
       </c>
       <c r="C21" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C21</f>
-        <v>36782.3174679213</v>
+        <v>55737.1828766041</v>
       </c>
       <c r="D21" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D21</f>
-        <v>29578.015</v>
+        <v>35701.755</v>
       </c>
       <c r="E21" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F21</f>
@@ -7225,11 +7225,11 @@
       </c>
       <c r="F21" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>17344.500865412</v>
+        <v>21426.5621233959</v>
       </c>
       <c r="G21" s="52" t="n">
         <f aca="false">G20+F21</f>
-        <v>-21981.4130291307</v>
+        <v>-329.207146965571</v>
       </c>
       <c r="H21" s="55" t="str">
         <f aca="false">IF(G21&gt;=0,"Sim","Não")</f>
@@ -7242,15 +7242,15 @@
       </c>
       <c r="B22" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B22</f>
-        <v>89265</v>
+        <v>120259</v>
       </c>
       <c r="C22" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C22</f>
-        <v>39663.1104350631</v>
+        <v>59916.8317975888</v>
       </c>
       <c r="D22" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D22</f>
-        <v>30745.65</v>
+        <v>37254.39</v>
       </c>
       <c r="E22" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F22</f>
@@ -7258,15 +7258,15 @@
       </c>
       <c r="F22" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>18856.2395649369</v>
+        <v>23087.7782024112</v>
       </c>
       <c r="G22" s="52" t="n">
         <f aca="false">G21+F22</f>
-        <v>-3125.17346419381</v>
+        <v>22758.5710554456</v>
       </c>
       <c r="H22" s="55" t="str">
         <f aca="false">IF(G22&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7275,15 +7275,15 @@
       </c>
       <c r="B23" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B23</f>
-        <v>91659</v>
+        <v>122653</v>
       </c>
       <c r="C23" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C23</f>
-        <v>40460.3358834631</v>
+        <v>60848.7212746378</v>
       </c>
       <c r="D23" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D23</f>
-        <v>31248.39</v>
+        <v>37757.13</v>
       </c>
       <c r="E23" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F23</f>
@@ -7291,11 +7291,11 @@
       </c>
       <c r="F23" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>19950.2741165369</v>
+        <v>24047.1487253622</v>
       </c>
       <c r="G23" s="52" t="n">
         <f aca="false">G22+F23</f>
-        <v>16825.1006523431</v>
+        <v>46805.7197808079</v>
       </c>
       <c r="H23" s="55" t="str">
         <f aca="false">IF(G23&gt;=0,"Sim","Não")</f>
@@ -7308,15 +7308,15 @@
       </c>
       <c r="B24" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B24</f>
-        <v>94053</v>
+        <v>135044</v>
       </c>
       <c r="C24" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C24</f>
-        <v>41285.1723624962</v>
+        <v>68407.3617410183</v>
       </c>
       <c r="D24" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D24</f>
-        <v>31751.13</v>
+        <v>40359.24</v>
       </c>
       <c r="E24" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F24</f>
@@ -7324,11 +7324,11 @@
       </c>
       <c r="F24" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>21016.6976375038</v>
+        <v>26277.3982589817</v>
       </c>
       <c r="G24" s="52" t="n">
         <f aca="false">G23+F24</f>
-        <v>37841.7982898469</v>
+        <v>73083.1180397896</v>
       </c>
       <c r="H24" s="55" t="str">
         <f aca="false">IF(G24&gt;=0,"Sim","Não")</f>
@@ -7341,15 +7341,15 @@
       </c>
       <c r="B25" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B25</f>
-        <v>96447</v>
+        <v>137438</v>
       </c>
       <c r="C25" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C25</f>
-        <v>42092.6402743522</v>
+        <v>69293.6477053512</v>
       </c>
       <c r="D25" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D25</f>
-        <v>32253.87</v>
+        <v>40861.98</v>
       </c>
       <c r="E25" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F25</f>
@@ -7357,11 +7357,11 @@
       </c>
       <c r="F25" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>22100.4897256478</v>
+        <v>27282.3722946488</v>
       </c>
       <c r="G25" s="52" t="n">
         <f aca="false">G24+F25</f>
-        <v>59942.2880154947</v>
+        <v>100365.490334438</v>
       </c>
       <c r="H25" s="55" t="str">
         <f aca="false">IF(G25&gt;=0,"Sim","Não")</f>
@@ -7374,15 +7374,15 @@
       </c>
       <c r="B26" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B26</f>
-        <v>108838</v>
+        <v>139832</v>
       </c>
       <c r="C26" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C26</f>
-        <v>49543.0975411268</v>
+        <v>70144.195380357</v>
       </c>
       <c r="D26" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D26</f>
-        <v>34855.98</v>
+        <v>41364.72</v>
       </c>
       <c r="E26" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F26</f>
@@ -7390,11 +7390,11 @@
       </c>
       <c r="F26" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>24438.9224588732</v>
+        <v>28323.084619643</v>
       </c>
       <c r="G26" s="52" t="n">
         <f aca="false">G25+F26</f>
-        <v>84381.2104743679</v>
+        <v>128688.574954081</v>
       </c>
       <c r="H26" s="55" t="str">
         <f aca="false">IF(G26&gt;=0,"Sim","Não")</f>
@@ -7407,15 +7407,15 @@
       </c>
       <c r="B27" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B27</f>
-        <v>111232</v>
+        <v>142226</v>
       </c>
       <c r="C27" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C27</f>
-        <v>50332.999998654</v>
+        <v>70959.0161541562</v>
       </c>
       <c r="D27" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D27</f>
-        <v>35358.72</v>
+        <v>41867.46</v>
       </c>
       <c r="E27" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F27</f>
@@ -7423,11 +7423,11 @@
       </c>
       <c r="F27" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>25540.280001346</v>
+        <v>29399.5238458438</v>
       </c>
       <c r="G27" s="52" t="n">
         <f aca="false">G26+F27</f>
-        <v>109921.490475714</v>
+        <v>158088.098799925</v>
       </c>
       <c r="H27" s="55" t="str">
         <f aca="false">IF(G27&gt;=0,"Sim","Não")</f>
@@ -7440,15 +7440,15 @@
       </c>
       <c r="B28" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B28</f>
-        <v>100462.833333333</v>
+        <v>139620.5</v>
       </c>
       <c r="C28" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C28</f>
-        <v>42320.3835692858</v>
+        <v>68507.3775253362</v>
       </c>
       <c r="D28" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D28</f>
-        <v>33097.195</v>
+        <v>41320.305</v>
       </c>
       <c r="E28" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F28</f>
@@ -7456,11 +7456,11 @@
       </c>
       <c r="F28" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>25045.2547640475</v>
+        <v>29792.8174746638</v>
       </c>
       <c r="G28" s="52" t="n">
         <f aca="false">G27+F28</f>
-        <v>134966.745239761</v>
+        <v>187880.916274589</v>
       </c>
       <c r="H28" s="55" t="str">
         <f aca="false">IF(G28&gt;=0,"Sim","Não")</f>
@@ -7473,15 +7473,15 @@
       </c>
       <c r="B29" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!B29</f>
-        <v>112853.833333333</v>
+        <v>142014.5</v>
       </c>
       <c r="C29" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!C29</f>
-        <v>49744.8745976521</v>
+        <v>69283.6107304242</v>
       </c>
       <c r="D29" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!D29</f>
-        <v>35699.305</v>
+        <v>41823.045</v>
       </c>
       <c r="E29" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!F29</f>
@@ -7489,11 +7489,11 @@
       </c>
       <c r="F29" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>27409.6537356813</v>
+        <v>30907.8442695758</v>
       </c>
       <c r="G29" s="52" t="n">
         <f aca="false">G28+F29</f>
-        <v>162376.398975443</v>
+        <v>218788.760544165</v>
       </c>
       <c r="H29" s="55" t="str">
         <f aca="false">IF(G29&gt;=0,"Sim","Não")</f>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="F33" s="58" t="n">
         <f aca="false">IFERROR(INDEX(A5:A29,MATCH("Sim",H5:H29,0)),"Não recupera")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G33" s="57" t="s">
         <v>233</v>
@@ -7818,7 +7818,7 @@
       </c>
       <c r="B17" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>368.560833333333</v>
+        <v>762.727500000001</v>
       </c>
       <c r="C17" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A17</f>
@@ -7826,11 +7826,11 @@
       </c>
       <c r="D17" s="51" t="n">
         <f aca="false">B17*C17</f>
-        <v>330.977398930366</v>
+        <v>684.949515008135</v>
       </c>
       <c r="E17" s="52" t="n">
         <f aca="false">E16+D17</f>
-        <v>-124424.020562105</v>
+        <v>-124070.048446028</v>
       </c>
       <c r="F17" s="55" t="str">
         <f aca="false">IF(E17&gt;=0,"Sim","Não")</f>
@@ -7843,7 +7843,7 @@
       </c>
       <c r="B18" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>2178.95687805391</v>
+        <v>2552.70057627762</v>
       </c>
       <c r="C18" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A18</f>
@@ -7851,11 +7851,11 @@
       </c>
       <c r="D18" s="51" t="n">
         <f aca="false">B18*C18</f>
-        <v>1921.99676589479</v>
+        <v>2251.66560261867</v>
       </c>
       <c r="E18" s="52" t="n">
         <f aca="false">E17+D18</f>
-        <v>-122502.023796211</v>
+        <v>-121818.382843409</v>
       </c>
       <c r="F18" s="55" t="str">
         <f aca="false">IF(E18&gt;=0,"Sim","Não")</f>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="B19" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>3816.02222603415</v>
+        <v>4559.67653753027</v>
       </c>
       <c r="C19" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A19</f>
@@ -7876,11 +7876,11 @@
       </c>
       <c r="D19" s="51" t="n">
         <f aca="false">B19*C19</f>
-        <v>3306.20495253736</v>
+        <v>3950.5076903124</v>
       </c>
       <c r="E19" s="52" t="n">
         <f aca="false">E18+D19</f>
-        <v>-119195.818843673</v>
+        <v>-117867.875153097</v>
       </c>
       <c r="F19" s="55" t="str">
         <f aca="false">IF(E19&gt;=0,"Sim","Não")</f>
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B20" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>7097.27217850077</v>
+        <v>7816.91318552533</v>
       </c>
       <c r="C20" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A20</f>
@@ -7901,11 +7901,11 @@
       </c>
       <c r="D20" s="51" t="n">
         <f aca="false">B20*C20</f>
-        <v>6039.83670085886</v>
+        <v>6652.25708665673</v>
       </c>
       <c r="E20" s="52" t="n">
         <f aca="false">E19+D20</f>
-        <v>-113155.982142814</v>
+        <v>-111215.61806644</v>
       </c>
       <c r="F20" s="55" t="str">
         <f aca="false">IF(E20&gt;=0,"Sim","Não")</f>
@@ -7918,7 +7918,7 @@
       </c>
       <c r="B21" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>7245.71718252431</v>
+        <v>8333.57875477045</v>
       </c>
       <c r="C21" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A21</f>
@@ -7926,11 +7926,11 @@
       </c>
       <c r="D21" s="51" t="n">
         <f aca="false">B21*C21</f>
-        <v>6056.61508901444</v>
+        <v>6965.94658060456</v>
       </c>
       <c r="E21" s="52" t="n">
         <f aca="false">E20+D21</f>
-        <v>-107099.3670538</v>
+        <v>-104249.671485835</v>
       </c>
       <c r="F21" s="55" t="str">
         <f aca="false">IF(E21&gt;=0,"Sim","Não")</f>
@@ -7943,7 +7943,7 @@
       </c>
       <c r="B22" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>10510.1917088394</v>
+        <v>11562.1018220183</v>
       </c>
       <c r="C22" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A22</f>
@@ -7951,11 +7951,11 @@
       </c>
       <c r="D22" s="51" t="n">
         <f aca="false">B22*C22</f>
-        <v>8629.27070023434</v>
+        <v>9492.92926807002</v>
       </c>
       <c r="E22" s="52" t="n">
         <f aca="false">E21+D22</f>
-        <v>-98470.0963535656</v>
+        <v>-94756.7422177652</v>
       </c>
       <c r="F22" s="55" t="str">
         <f aca="false">IF(E22&gt;=0,"Sim","Não")</f>
@@ -7968,7 +7968,7 @@
       </c>
       <c r="B23" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>10216.5802377799</v>
+        <v>11226.7223367435</v>
       </c>
       <c r="C23" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A23</f>
@@ -7976,11 +7976,11 @@
       </c>
       <c r="D23" s="51" t="n">
         <f aca="false">B23*C23</f>
-        <v>8239.17761111282</v>
+        <v>9053.80833608344</v>
       </c>
       <c r="E23" s="52" t="n">
         <f aca="false">E22+D23</f>
-        <v>-90230.9187424528</v>
+        <v>-85702.9338816818</v>
       </c>
       <c r="F23" s="55" t="str">
         <f aca="false">IF(E23&gt;=0,"Sim","Não")</f>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="B24" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>13832.9830981497</v>
+        <v>17923.346960382</v>
       </c>
       <c r="C24" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A24</f>
@@ -8001,11 +8001,11 @@
       </c>
       <c r="D24" s="51" t="n">
         <f aca="false">B24*C24</f>
-        <v>10957.4379677169</v>
+        <v>14197.5133706714</v>
       </c>
       <c r="E24" s="52" t="n">
         <f aca="false">E23+D24</f>
-        <v>-79273.4807747359</v>
+        <v>-71505.4205110103</v>
       </c>
       <c r="F24" s="55" t="str">
         <f aca="false">IF(E24&gt;=0,"Sim","Não")</f>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="B25" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>14824.0390586497</v>
+        <v>18752.818108067</v>
       </c>
       <c r="C25" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A25</f>
@@ -8026,11 +8026,11 @@
       </c>
       <c r="D25" s="51" t="n">
         <f aca="false">B25*C25</f>
-        <v>11533.857583567</v>
+        <v>14590.6478317578</v>
       </c>
       <c r="E25" s="52" t="n">
         <f aca="false">E24+D25</f>
-        <v>-67739.6231911689</v>
+        <v>-56914.7726792525</v>
       </c>
       <c r="F25" s="55" t="str">
         <f aca="false">IF(E25&gt;=0,"Sim","Não")</f>
@@ -8043,7 +8043,7 @@
       </c>
       <c r="B26" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>16278.2027035919</v>
+        <v>20448.0849483241</v>
       </c>
       <c r="C26" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A26</f>
@@ -8051,11 +8051,11 @@
       </c>
       <c r="D26" s="51" t="n">
         <f aca="false">B26*C26</f>
-        <v>12440.256809103</v>
+        <v>15626.9971964027</v>
       </c>
       <c r="E26" s="52" t="n">
         <f aca="false">E25+D26</f>
-        <v>-55299.3663820659</v>
+        <v>-41287.7754828498</v>
       </c>
       <c r="F26" s="55" t="str">
         <f aca="false">IF(E26&gt;=0,"Sim","Não")</f>
@@ -8068,7 +8068,7 @@
       </c>
       <c r="B27" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>17344.500865412</v>
+        <v>21426.5621233959</v>
       </c>
       <c r="C27" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A27</f>
@@ -8076,11 +8076,11 @@
       </c>
       <c r="D27" s="51" t="n">
         <f aca="false">B27*C27</f>
-        <v>13019.6574944928</v>
+        <v>16083.8586417551</v>
       </c>
       <c r="E27" s="52" t="n">
         <f aca="false">E26+D27</f>
-        <v>-42279.7088875731</v>
+        <v>-25203.9168410947</v>
       </c>
       <c r="F27" s="55" t="str">
         <f aca="false">IF(E27&gt;=0,"Sim","Não")</f>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="B28" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>18856.2395649369</v>
+        <v>23087.7782024112</v>
       </c>
       <c r="C28" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A28</f>
@@ -8101,11 +8101,11 @@
       </c>
       <c r="D28" s="51" t="n">
         <f aca="false">B28*C28</f>
-        <v>13902.9736568</v>
+        <v>17022.9472868515</v>
       </c>
       <c r="E28" s="52" t="n">
         <f aca="false">E27+D28</f>
-        <v>-28376.7352307731</v>
+        <v>-8180.96955424323</v>
       </c>
       <c r="F28" s="55" t="str">
         <f aca="false">IF(E28&gt;=0,"Sim","Não")</f>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="B29" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>19950.2741165369</v>
+        <v>24047.1487253622</v>
       </c>
       <c r="C29" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A29</f>
@@ -8126,15 +8126,15 @@
       </c>
       <c r="D29" s="51" t="n">
         <f aca="false">B29*C29</f>
-        <v>14448.2863234579</v>
+        <v>17415.3040713768</v>
       </c>
       <c r="E29" s="52" t="n">
         <f aca="false">E28+D29</f>
-        <v>-13928.4489073152</v>
+        <v>9234.33451713362</v>
       </c>
       <c r="F29" s="55" t="str">
         <f aca="false">IF(E29&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8143,7 +8143,7 @@
       </c>
       <c r="B30" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>21016.6976375038</v>
+        <v>26277.3982589817</v>
       </c>
       <c r="C30" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A30</f>
@@ -8151,11 +8151,11 @@
       </c>
       <c r="D30" s="51" t="n">
         <f aca="false">B30*C30</f>
-        <v>14950.1933019155</v>
+        <v>18692.3840376406</v>
       </c>
       <c r="E30" s="52" t="n">
         <f aca="false">E29+D30</f>
-        <v>1021.74439460032</v>
+        <v>27926.7185547742</v>
       </c>
       <c r="F30" s="55" t="str">
         <f aca="false">IF(E30&gt;=0,"Sim","Não")</f>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="B31" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>22100.4897256478</v>
+        <v>27282.3722946488</v>
       </c>
       <c r="C31" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A31</f>
@@ -8176,11 +8176,11 @@
       </c>
       <c r="D31" s="51" t="n">
         <f aca="false">B31*C31</f>
-        <v>15441.841440735</v>
+        <v>19062.4765482983</v>
       </c>
       <c r="E31" s="52" t="n">
         <f aca="false">E30+D31</f>
-        <v>16463.5858353353</v>
+        <v>46989.1951030726</v>
       </c>
       <c r="F31" s="55" t="str">
         <f aca="false">IF(E31&gt;=0,"Sim","Não")</f>
@@ -8193,7 +8193,7 @@
       </c>
       <c r="B32" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>24438.9224588732</v>
+        <v>28323.084619643</v>
       </c>
       <c r="C32" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A32</f>
@@ -8201,11 +8201,11 @@
       </c>
       <c r="D32" s="51" t="n">
         <f aca="false">B32*C32</f>
-        <v>16772.3572549375</v>
+        <v>19438.0457895353</v>
       </c>
       <c r="E32" s="52" t="n">
         <f aca="false">E31+D32</f>
-        <v>33235.9430902729</v>
+        <v>66427.2408926079</v>
       </c>
       <c r="F32" s="55" t="str">
         <f aca="false">IF(E32&gt;=0,"Sim","Não")</f>
@@ -8218,7 +8218,7 @@
       </c>
       <c r="B33" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>25540.280001346</v>
+        <v>29399.5238458438</v>
       </c>
       <c r="C33" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A33</f>
@@ -8226,11 +8226,11 @@
       </c>
       <c r="D33" s="51" t="n">
         <f aca="false">B33*C33</f>
-        <v>17216.805162625</v>
+        <v>19818.3369133448</v>
       </c>
       <c r="E33" s="52" t="n">
         <f aca="false">E32+D33</f>
-        <v>50452.7482528978</v>
+        <v>86245.5778059527</v>
       </c>
       <c r="F33" s="55" t="str">
         <f aca="false">IF(E33&gt;=0,"Sim","Não")</f>
@@ -8243,7 +8243,7 @@
       </c>
       <c r="B34" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>25045.2547640475</v>
+        <v>29792.8174746638</v>
       </c>
       <c r="C34" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A34</f>
@@ -8251,11 +8251,11 @@
       </c>
       <c r="D34" s="51" t="n">
         <f aca="false">B34*C34</f>
-        <v>16583.1574371831</v>
+        <v>19726.6503109735</v>
       </c>
       <c r="E34" s="52" t="n">
         <f aca="false">E33+D34</f>
-        <v>67035.9056900809</v>
+        <v>105972.228116926</v>
       </c>
       <c r="F34" s="55" t="str">
         <f aca="false">IF(E34&gt;=0,"Sim","Não")</f>
@@ -8268,7 +8268,7 @@
       </c>
       <c r="B35" s="51" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>27409.6537356813</v>
+        <v>30907.8442695758</v>
       </c>
       <c r="C35" s="62" t="n">
         <f aca="false">1/(1+$B$7)^A35</f>
@@ -8276,11 +8276,11 @@
       </c>
       <c r="D35" s="51" t="n">
         <f aca="false">B35*C35</f>
-        <v>17826.257632467</v>
+        <v>20101.3555343235</v>
       </c>
       <c r="E35" s="52" t="n">
         <f aca="false">E34+D35</f>
-        <v>84862.1633225479</v>
+        <v>126073.58365125</v>
       </c>
       <c r="F35" s="55" t="str">
         <f aca="false">IF(E35&gt;=0,"Sim","Não")</f>
@@ -8304,7 +8304,7 @@
       </c>
       <c r="B38" s="63" t="n">
         <f aca="false">SUM(D11:D35)</f>
-        <v>84862.163322548</v>
+        <v>126073.58365125</v>
       </c>
       <c r="C38" s="64" t="str">
         <f aca="false">IF(B38&gt;0,"VIÁVEL: o projeto gera mais do que a taxa exigida",IF(B38&lt;0,"INVIÁVEL: o projeto rende menos que a taxa exigida","EQUILÍBRIO: rende exatamente a taxa exigida"))</f>
@@ -8317,7 +8317,7 @@
       </c>
       <c r="B39" s="65" t="n">
         <f aca="false">IFERROR(IRR(B11:B35),"Não calculável")</f>
-        <v>0.0499656736839225</v>
+        <v>0.0615783311983349</v>
       </c>
       <c r="C39" s="64" t="str">
         <f aca="false">IF(ISNUMBER(B39),IF(B39&gt;B7,"VIÁVEL: TIR maior que a taxa de desconto","INVIÁVEL: TIR menor ou igual à taxa de desconto"),"Sem TIR: o fluxo precisa ter valores negativos E positivos")</f>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="B40" s="65" t="n">
         <f aca="false">IF(ISNUMBER(B39),IF(B6="Mensal",(1+B39)^12-1,B39),"Não calculável")</f>
-        <v>0.795151936890566</v>
+        <v>1.04844610560403</v>
       </c>
       <c r="C40" s="64" t="str">
         <f aca="false">"Compare com a taxa anual de "&amp;ROUND(B5*100,2)&amp;"%"</f>
@@ -8356,11 +8356,11 @@
       </c>
       <c r="B42" s="65" t="n">
         <f aca="false">IF(B41=0,"-",B38/B41)</f>
-        <v>0.831981993358313</v>
+        <v>1.23601552599264</v>
       </c>
       <c r="C42" s="64" t="str">
         <f aca="false">"Para cada R$ 100 de investimento inicial, o projeto gera R$ "&amp;IF(ISNUMBER(B42),ROUND(B42*100,2),"-")&amp;" de VPL acima da taxa exigida"</f>
-        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 83.2 de VPL acima da taxa exigida</v>
+        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 123.6 de VPL acima da taxa exigida</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8369,7 +8369,7 @@
       </c>
       <c r="B43" s="66" t="n">
         <f aca="false">'Necessidade de Caixa e Payback'!F33</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C43" s="64" t="str">
         <f aca="false">"Período em que o saldo acumulado (sem descontar) fica positivo"</f>
@@ -8382,7 +8382,7 @@
       </c>
       <c r="B44" s="66" t="n">
         <f aca="false">IFERROR(INDEX(A11:A35,MATCH("Sim",F11:F35,0)),"Não recupera")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C44" s="64" t="str">
         <f aca="false">"Período em que o VP acumulado fica positivo"</f>

</xml_diff>